<commit_message>
src code ready for detect_language and lemmatize_str
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28814"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/464195223dcae84f/Dokumente/OECD/RAnalysis/PRESS/data/keywords/review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_AD4DB114E441178AC67DF4704E97EB86683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{429A4230-4344-409D-87B1-23333E8C3D89}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="11_AD4DB114E441178AC67DF4704E97EB86683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CBB7C5F-5F72-43CB-82E7-D5742DE9605C}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -40,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="455">
   <si>
     <t>en</t>
   </si>
@@ -135,9 +133,6 @@
     <t>registro civil</t>
   </si>
   <si>
-    <t>Melderegister</t>
-  </si>
-  <si>
     <t>land register</t>
   </si>
   <si>
@@ -165,9 +160,6 @@
     <t>sdg indicator</t>
   </si>
   <si>
-    <t>Indicateur sdg</t>
-  </si>
-  <si>
     <t>indicador sdg</t>
   </si>
   <si>
@@ -894,9 +886,6 @@
     <t>seguimiento de los prsp</t>
   </si>
   <si>
-    <t>prsp-überwachung</t>
-  </si>
-  <si>
     <t>data revolution</t>
   </si>
   <si>
@@ -915,12 +904,6 @@
     <t>diseminar datos</t>
   </si>
   <si>
-    <t>usuario de estadísticas</t>
-  </si>
-  <si>
-    <t>productor de estadísticas</t>
-  </si>
-  <si>
     <t>es</t>
   </si>
   <si>
@@ -960,21 +943,9 @@
     <t>ckan</t>
   </si>
   <si>
-    <t>lfs questionnaire</t>
-  </si>
-  <si>
     <t>enquête emploi</t>
   </si>
   <si>
-    <t xml:space="preserve">lfs </t>
-  </si>
-  <si>
-    <t>EDS</t>
-  </si>
-  <si>
-    <t>Arbeitskräfteerhebung</t>
-  </si>
-  <si>
     <t>IPC</t>
   </si>
   <si>
@@ -1414,13 +1385,31 @@
   </si>
   <si>
     <t>SDSR</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Unternehmensregister</t>
+  </si>
+  <si>
+    <t>Datenwissenschaften</t>
+  </si>
+  <si>
+    <t>Indicateur odd</t>
+  </si>
+  <si>
+    <t>prsp-Überwachung</t>
+  </si>
+  <si>
+    <t>lfs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1759,1055 +1748,1278 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D77"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:E76"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.140625" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="2" max="2" width="18.86328125" customWidth="1"/>
+    <col min="3" max="3" width="32.1328125" customWidth="1"/>
+    <col min="4" max="4" width="31.265625" customWidth="1"/>
+    <col min="5" max="5" width="30.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>26</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>33</v>
       </c>
-      <c r="C9" t="s">
+      <c r="E9" t="s">
         <v>34</v>
       </c>
-      <c r="D9" t="s">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
+      <c r="C10" t="s">
         <v>36</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
         <v>37</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
         <v>38</v>
       </c>
-      <c r="D10" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+      <c r="C11" t="s">
+        <v>452</v>
+      </c>
+      <c r="D11" t="s">
         <v>40</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>42</v>
       </c>
-      <c r="D11" t="s">
+      <c r="C12" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+      <c r="D12" t="s">
         <v>44</v>
       </c>
-      <c r="B12" t="s">
+      <c r="E12" t="s">
         <v>45</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
         <v>46</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C13" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
+      <c r="D13" t="s">
         <v>48</v>
       </c>
-      <c r="B13" t="s">
+      <c r="E13" t="s">
         <v>49</v>
       </c>
-      <c r="C13" t="s">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
         <v>50</v>
       </c>
-      <c r="D13" t="s">
+      <c r="C14" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="D14" t="s">
         <v>52</v>
       </c>
-      <c r="B14" t="s">
+      <c r="E14" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>16</v>
+      </c>
+      <c r="E19" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>90</v>
+      </c>
+      <c r="C25" t="s">
+        <v>91</v>
+      </c>
+      <c r="D25" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A26">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" t="s">
+        <v>95</v>
+      </c>
+      <c r="D26" t="s">
+        <v>96</v>
+      </c>
+      <c r="E26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A27">
+        <v>24</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" t="s">
+        <v>98</v>
+      </c>
+      <c r="D27" t="s">
+        <v>99</v>
+      </c>
+      <c r="E27" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A28">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" t="s">
+        <v>102</v>
+      </c>
+      <c r="D28" t="s">
+        <v>103</v>
+      </c>
+      <c r="E28" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A29">
+        <v>26</v>
+      </c>
+      <c r="B29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" t="s">
+        <v>106</v>
+      </c>
+      <c r="D29" t="s">
+        <v>107</v>
+      </c>
+      <c r="E29" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A30">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" t="s">
+        <v>111</v>
+      </c>
+      <c r="E30" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A31">
+        <v>28</v>
+      </c>
+      <c r="B31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" t="s">
+        <v>114</v>
+      </c>
+      <c r="D31" t="s">
+        <v>115</v>
+      </c>
+      <c r="E31" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A32">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" t="s">
+        <v>119</v>
+      </c>
+      <c r="E32" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A33">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>121</v>
+      </c>
+      <c r="C33" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E33" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" t="s">
+        <v>126</v>
+      </c>
+      <c r="D34" t="s">
+        <v>127</v>
+      </c>
+      <c r="E34" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35">
+        <v>32</v>
+      </c>
+      <c r="B35" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" t="s">
+        <v>130</v>
+      </c>
+      <c r="D35" t="s">
+        <v>131</v>
+      </c>
+      <c r="E35" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A36">
+        <v>33</v>
+      </c>
+      <c r="B36" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A37">
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>137</v>
+      </c>
+      <c r="C37" t="s">
+        <v>138</v>
+      </c>
+      <c r="D37" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A38">
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>141</v>
+      </c>
+      <c r="C38" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" t="s">
+        <v>143</v>
+      </c>
+      <c r="E38" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A39">
+        <v>36</v>
+      </c>
+      <c r="B39" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" t="s">
+        <v>146</v>
+      </c>
+      <c r="D39" t="s">
+        <v>147</v>
+      </c>
+      <c r="E39" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A40">
+        <v>37</v>
+      </c>
+      <c r="B40" t="s">
+        <v>149</v>
+      </c>
+      <c r="C40" t="s">
+        <v>150</v>
+      </c>
+      <c r="D40" t="s">
+        <v>151</v>
+      </c>
+      <c r="E40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A41">
+        <v>37</v>
+      </c>
+      <c r="D41" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A42">
+        <v>38</v>
+      </c>
+      <c r="B42" t="s">
+        <v>153</v>
+      </c>
+      <c r="C42" t="s">
+        <v>154</v>
+      </c>
+      <c r="D42" t="s">
+        <v>155</v>
+      </c>
+      <c r="E42" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A43">
+        <v>38</v>
+      </c>
+      <c r="D43" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A44">
+        <v>39</v>
+      </c>
+      <c r="B44" t="s">
+        <v>157</v>
+      </c>
+      <c r="C44" t="s">
+        <v>158</v>
+      </c>
+      <c r="D44" t="s">
+        <v>159</v>
+      </c>
+      <c r="E44" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A45">
+        <v>40</v>
+      </c>
+      <c r="B45" t="s">
+        <v>161</v>
+      </c>
+      <c r="C45" t="s">
+        <v>162</v>
+      </c>
+      <c r="D45" t="s">
+        <v>163</v>
+      </c>
+      <c r="E45" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A46">
+        <v>41</v>
+      </c>
+      <c r="B46" t="s">
+        <v>165</v>
+      </c>
+      <c r="C46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" t="s">
+        <v>167</v>
+      </c>
+      <c r="E46" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A47">
+        <v>42</v>
+      </c>
+      <c r="B47" t="s">
+        <v>169</v>
+      </c>
+      <c r="C47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D47" t="s">
+        <v>171</v>
+      </c>
+      <c r="E47" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A48">
+        <v>43</v>
+      </c>
+      <c r="B48" t="s">
+        <v>173</v>
+      </c>
+      <c r="C48" t="s">
+        <v>174</v>
+      </c>
+      <c r="D48" t="s">
+        <v>175</v>
+      </c>
+      <c r="E48" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A49">
+        <v>44</v>
+      </c>
+      <c r="B49" t="s">
+        <v>177</v>
+      </c>
+      <c r="C49" t="s">
+        <v>178</v>
+      </c>
+      <c r="D49" t="s">
+        <v>179</v>
+      </c>
+      <c r="E49" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A50">
+        <v>45</v>
+      </c>
+      <c r="B50" t="s">
+        <v>181</v>
+      </c>
+      <c r="C50" t="s">
+        <v>182</v>
+      </c>
+      <c r="D50" t="s">
+        <v>183</v>
+      </c>
+      <c r="E50" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A51">
+        <v>46</v>
+      </c>
+      <c r="B51" t="s">
+        <v>185</v>
+      </c>
+      <c r="C51" t="s">
+        <v>186</v>
+      </c>
+      <c r="D51" t="s">
+        <v>187</v>
+      </c>
+      <c r="E51" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A52">
+        <v>47</v>
+      </c>
+      <c r="B52" t="s">
+        <v>189</v>
+      </c>
+      <c r="C52" t="s">
+        <v>190</v>
+      </c>
+      <c r="D52" t="s">
+        <v>191</v>
+      </c>
+      <c r="E52" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A53">
+        <v>48</v>
+      </c>
+      <c r="B53" t="s">
+        <v>193</v>
+      </c>
+      <c r="C53" t="s">
+        <v>194</v>
+      </c>
+      <c r="D53" t="s">
+        <v>195</v>
+      </c>
+      <c r="E53" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A54">
+        <v>49</v>
+      </c>
+      <c r="B54" t="s">
+        <v>197</v>
+      </c>
+      <c r="C54" t="s">
+        <v>198</v>
+      </c>
+      <c r="D54" t="s">
+        <v>199</v>
+      </c>
+      <c r="E54" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A55">
+        <v>50</v>
+      </c>
+      <c r="B55" t="s">
+        <v>201</v>
+      </c>
+      <c r="C55" t="s">
+        <v>190</v>
+      </c>
+      <c r="D55" t="s">
+        <v>202</v>
+      </c>
+      <c r="E55" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A56">
+        <v>51</v>
+      </c>
+      <c r="B56" t="s">
+        <v>204</v>
+      </c>
+      <c r="C56" t="s">
+        <v>194</v>
+      </c>
+      <c r="D56" t="s">
+        <v>205</v>
+      </c>
+      <c r="E56" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A57">
+        <v>52</v>
+      </c>
+      <c r="B57" t="s">
+        <v>207</v>
+      </c>
+      <c r="C57" t="s">
+        <v>208</v>
+      </c>
+      <c r="D57" t="s">
+        <v>209</v>
+      </c>
+      <c r="E57" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A58">
         <v>53</v>
       </c>
-      <c r="C14" t="s">
+      <c r="B58" t="s">
+        <v>211</v>
+      </c>
+      <c r="C58" t="s">
+        <v>212</v>
+      </c>
+      <c r="D58" t="s">
+        <v>213</v>
+      </c>
+      <c r="E58" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A59">
         <v>54</v>
       </c>
-      <c r="D14" t="s">
+      <c r="B59" t="s">
+        <v>215</v>
+      </c>
+      <c r="C59" t="s">
+        <v>216</v>
+      </c>
+      <c r="D59" t="s">
+        <v>217</v>
+      </c>
+      <c r="E59" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A60">
         <v>55</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+      <c r="B60" t="s">
+        <v>219</v>
+      </c>
+      <c r="C60" t="s">
+        <v>220</v>
+      </c>
+      <c r="D60" t="s">
+        <v>221</v>
+      </c>
+      <c r="E60" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A61">
         <v>56</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B61" t="s">
+        <v>223</v>
+      </c>
+      <c r="C61" t="s">
+        <v>224</v>
+      </c>
+      <c r="D61" t="s">
+        <v>225</v>
+      </c>
+      <c r="E61" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A62">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B62" t="s">
+        <v>227</v>
+      </c>
+      <c r="C62" t="s">
+        <v>228</v>
+      </c>
+      <c r="D62" t="s">
+        <v>229</v>
+      </c>
+      <c r="E62" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A63">
         <v>58</v>
       </c>
-      <c r="D15" t="s">
+      <c r="B63" t="s">
+        <v>231</v>
+      </c>
+      <c r="C63" t="s">
+        <v>232</v>
+      </c>
+      <c r="D63" t="s">
+        <v>233</v>
+      </c>
+      <c r="E63" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A64">
         <v>59</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="B64" t="s">
+        <v>235</v>
+      </c>
+      <c r="C64" t="s">
+        <v>236</v>
+      </c>
+      <c r="D64" t="s">
+        <v>237</v>
+      </c>
+      <c r="E64" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A65">
         <v>60</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B65" t="s">
+        <v>239</v>
+      </c>
+      <c r="C65" t="s">
+        <v>240</v>
+      </c>
+      <c r="D65" t="s">
+        <v>241</v>
+      </c>
+      <c r="E65" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A66">
         <v>61</v>
       </c>
-      <c r="C16" t="s">
+      <c r="B66" t="s">
+        <v>243</v>
+      </c>
+      <c r="C66" t="s">
+        <v>244</v>
+      </c>
+      <c r="D66" t="s">
+        <v>245</v>
+      </c>
+      <c r="E66" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A67">
         <v>62</v>
       </c>
-      <c r="D16" t="s">
+      <c r="B67" t="s">
+        <v>247</v>
+      </c>
+      <c r="C67" t="s">
+        <v>248</v>
+      </c>
+      <c r="D67" t="s">
+        <v>249</v>
+      </c>
+      <c r="E67" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A68">
         <v>63</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="B68" t="s">
+        <v>251</v>
+      </c>
+      <c r="C68" t="s">
+        <v>252</v>
+      </c>
+      <c r="D68" t="s">
+        <v>253</v>
+      </c>
+      <c r="E68" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A69">
         <v>64</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B69" t="s">
+        <v>255</v>
+      </c>
+      <c r="C69" t="s">
+        <v>256</v>
+      </c>
+      <c r="D69" t="s">
+        <v>257</v>
+      </c>
+      <c r="E69" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A70">
         <v>65</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B70" t="s">
+        <v>259</v>
+      </c>
+      <c r="C70" t="s">
+        <v>264</v>
+      </c>
+      <c r="D70" t="s">
+        <v>261</v>
+      </c>
+      <c r="E70" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A71">
         <v>66</v>
       </c>
-      <c r="D17" t="s">
+      <c r="B71" t="s">
+        <v>263</v>
+      </c>
+      <c r="C71" t="s">
+        <v>260</v>
+      </c>
+      <c r="D71" t="s">
+        <v>265</v>
+      </c>
+      <c r="E71" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A72">
         <v>67</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="B72" t="s">
+        <v>267</v>
+      </c>
+      <c r="C72" t="s">
+        <v>268</v>
+      </c>
+      <c r="D72" t="s">
+        <v>269</v>
+      </c>
+      <c r="E72" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A73">
         <v>68</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B73" t="s">
+        <v>271</v>
+      </c>
+      <c r="C73" t="s">
+        <v>272</v>
+      </c>
+      <c r="D73" t="s">
+        <v>273</v>
+      </c>
+      <c r="E73" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A74">
         <v>69</v>
       </c>
-      <c r="C18" t="s">
+      <c r="B74" t="s">
+        <v>275</v>
+      </c>
+      <c r="C74" t="s">
+        <v>276</v>
+      </c>
+      <c r="D74" t="s">
+        <v>277</v>
+      </c>
+      <c r="E74" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A75">
         <v>70</v>
       </c>
-      <c r="D18" t="s">
+      <c r="B75" t="s">
+        <v>279</v>
+      </c>
+      <c r="C75" t="s">
+        <v>280</v>
+      </c>
+      <c r="D75" t="s">
+        <v>281</v>
+      </c>
+      <c r="E75" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A76">
         <v>71</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B19" t="s">
-        <v>73</v>
-      </c>
-      <c r="C19" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" t="s">
-        <v>77</v>
-      </c>
-      <c r="C20" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" t="s">
-        <v>81</v>
-      </c>
-      <c r="C21" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C22" t="s">
-        <v>86</v>
-      </c>
-      <c r="D22" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
-        <v>88</v>
-      </c>
-      <c r="B23" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23" t="s">
-        <v>90</v>
-      </c>
-      <c r="D23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
-        <v>92</v>
-      </c>
-      <c r="B24" t="s">
-        <v>93</v>
-      </c>
-      <c r="C24" t="s">
-        <v>94</v>
-      </c>
-      <c r="D24" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
-        <v>96</v>
-      </c>
-      <c r="B25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" t="s">
-        <v>98</v>
-      </c>
-      <c r="D25" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>100</v>
-      </c>
-      <c r="B26" t="s">
-        <v>100</v>
-      </c>
-      <c r="C26" t="s">
-        <v>101</v>
-      </c>
-      <c r="D26" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
-        <v>103</v>
-      </c>
-      <c r="B27" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
-        <v>107</v>
-      </c>
-      <c r="B28" t="s">
-        <v>108</v>
-      </c>
-      <c r="C28" t="s">
-        <v>109</v>
-      </c>
-      <c r="D28" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
-        <v>111</v>
-      </c>
-      <c r="B29" t="s">
-        <v>112</v>
-      </c>
-      <c r="C29" t="s">
-        <v>113</v>
-      </c>
-      <c r="D29" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" t="s">
-        <v>116</v>
-      </c>
-      <c r="C30" t="s">
-        <v>117</v>
-      </c>
-      <c r="D30" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
-        <v>119</v>
-      </c>
-      <c r="B31" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" t="s">
-        <v>121</v>
-      </c>
-      <c r="D31" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" t="s">
-        <v>123</v>
-      </c>
-      <c r="B32" t="s">
-        <v>124</v>
-      </c>
-      <c r="C32" t="s">
-        <v>125</v>
-      </c>
-      <c r="D32" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" t="s">
-        <v>127</v>
-      </c>
-      <c r="B33" t="s">
-        <v>128</v>
-      </c>
-      <c r="C33" t="s">
-        <v>129</v>
-      </c>
-      <c r="D33" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>131</v>
-      </c>
-      <c r="B34" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" t="s">
-        <v>133</v>
-      </c>
-      <c r="D34" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>135</v>
-      </c>
-      <c r="B35" t="s">
-        <v>136</v>
-      </c>
-      <c r="C35" t="s">
-        <v>137</v>
-      </c>
-      <c r="D35" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>139</v>
-      </c>
-      <c r="B36" t="s">
-        <v>140</v>
-      </c>
-      <c r="C36" t="s">
-        <v>141</v>
-      </c>
-      <c r="D36" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" t="s">
-        <v>143</v>
-      </c>
-      <c r="B37" t="s">
-        <v>144</v>
-      </c>
-      <c r="C37" t="s">
-        <v>145</v>
-      </c>
-      <c r="D37" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>147</v>
-      </c>
-      <c r="B38" t="s">
-        <v>148</v>
-      </c>
-      <c r="C38" t="s">
-        <v>149</v>
-      </c>
-      <c r="D38" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>151</v>
-      </c>
-      <c r="B39" t="s">
-        <v>152</v>
-      </c>
-      <c r="C39" t="s">
-        <v>153</v>
-      </c>
-      <c r="D39" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>155</v>
-      </c>
-      <c r="B40" t="s">
-        <v>156</v>
-      </c>
-      <c r="C40" t="s">
-        <v>157</v>
-      </c>
-      <c r="D40" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>159</v>
-      </c>
-      <c r="B41" t="s">
-        <v>160</v>
-      </c>
-      <c r="C41" t="s">
-        <v>161</v>
-      </c>
-      <c r="D41" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" t="s">
-        <v>163</v>
-      </c>
-      <c r="B42" t="s">
-        <v>164</v>
-      </c>
-      <c r="C42" t="s">
-        <v>165</v>
-      </c>
-      <c r="D42" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" t="s">
-        <v>167</v>
-      </c>
-      <c r="B43" t="s">
-        <v>168</v>
-      </c>
-      <c r="C43" t="s">
-        <v>169</v>
-      </c>
-      <c r="D43" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>171</v>
-      </c>
-      <c r="B44" t="s">
-        <v>172</v>
-      </c>
-      <c r="C44" t="s">
-        <v>173</v>
-      </c>
-      <c r="D44" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" t="s">
-        <v>175</v>
-      </c>
-      <c r="B45" t="s">
-        <v>176</v>
-      </c>
-      <c r="C45" t="s">
-        <v>177</v>
-      </c>
-      <c r="D45" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" t="s">
-        <v>179</v>
-      </c>
-      <c r="B46" t="s">
-        <v>180</v>
-      </c>
-      <c r="C46" t="s">
-        <v>181</v>
-      </c>
-      <c r="D46" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" t="s">
-        <v>183</v>
-      </c>
-      <c r="B47" t="s">
-        <v>184</v>
-      </c>
-      <c r="C47" t="s">
-        <v>185</v>
-      </c>
-      <c r="D47" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4">
-      <c r="A48" t="s">
-        <v>187</v>
-      </c>
-      <c r="B48" t="s">
-        <v>188</v>
-      </c>
-      <c r="C48" t="s">
-        <v>189</v>
-      </c>
-      <c r="D48" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4">
-      <c r="A49" t="s">
-        <v>191</v>
-      </c>
-      <c r="B49" t="s">
-        <v>192</v>
-      </c>
-      <c r="C49" t="s">
-        <v>193</v>
-      </c>
-      <c r="D49" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4">
-      <c r="A50" t="s">
-        <v>195</v>
-      </c>
-      <c r="B50" t="s">
-        <v>196</v>
-      </c>
-      <c r="C50" t="s">
-        <v>197</v>
-      </c>
-      <c r="D50" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
-      <c r="A51" t="s">
-        <v>199</v>
-      </c>
-      <c r="B51" t="s">
-        <v>200</v>
-      </c>
-      <c r="C51" t="s">
-        <v>201</v>
-      </c>
-      <c r="D51" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4">
-      <c r="A52" t="s">
-        <v>203</v>
-      </c>
-      <c r="B52" t="s">
-        <v>192</v>
-      </c>
-      <c r="C52" t="s">
-        <v>204</v>
-      </c>
-      <c r="D52" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4">
-      <c r="A53" t="s">
-        <v>206</v>
-      </c>
-      <c r="B53" t="s">
-        <v>196</v>
-      </c>
-      <c r="C53" t="s">
-        <v>207</v>
-      </c>
-      <c r="D53" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" t="s">
-        <v>209</v>
-      </c>
-      <c r="B54" t="s">
-        <v>210</v>
-      </c>
-      <c r="C54" t="s">
-        <v>211</v>
-      </c>
-      <c r="D54" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" t="s">
-        <v>213</v>
-      </c>
-      <c r="B55" t="s">
-        <v>214</v>
-      </c>
-      <c r="C55" t="s">
-        <v>215</v>
-      </c>
-      <c r="D55" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4">
-      <c r="A56" t="s">
-        <v>217</v>
-      </c>
-      <c r="B56" t="s">
-        <v>218</v>
-      </c>
-      <c r="C56" t="s">
-        <v>219</v>
-      </c>
-      <c r="D56" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="A57" t="s">
-        <v>221</v>
-      </c>
-      <c r="B57" t="s">
-        <v>222</v>
-      </c>
-      <c r="C57" t="s">
-        <v>223</v>
-      </c>
-      <c r="D57" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4">
-      <c r="A58" t="s">
-        <v>225</v>
-      </c>
-      <c r="B58" t="s">
-        <v>226</v>
-      </c>
-      <c r="C58" t="s">
-        <v>227</v>
-      </c>
-      <c r="D58" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4">
-      <c r="A59" t="s">
-        <v>229</v>
-      </c>
-      <c r="B59" t="s">
-        <v>230</v>
-      </c>
-      <c r="C59" t="s">
-        <v>231</v>
-      </c>
-      <c r="D59" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="A60" t="s">
-        <v>233</v>
-      </c>
-      <c r="B60" t="s">
-        <v>234</v>
-      </c>
-      <c r="C60" t="s">
-        <v>235</v>
-      </c>
-      <c r="D60" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="A61" t="s">
-        <v>237</v>
-      </c>
-      <c r="B61" t="s">
-        <v>238</v>
-      </c>
-      <c r="C61" t="s">
-        <v>239</v>
-      </c>
-      <c r="D61" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" t="s">
-        <v>241</v>
-      </c>
-      <c r="B62" t="s">
-        <v>242</v>
-      </c>
-      <c r="C62" t="s">
-        <v>243</v>
-      </c>
-      <c r="D62" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="A63" t="s">
-        <v>245</v>
-      </c>
-      <c r="B63" t="s">
-        <v>246</v>
-      </c>
-      <c r="C63" t="s">
-        <v>247</v>
-      </c>
-      <c r="D63" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="A64" t="s">
-        <v>249</v>
-      </c>
-      <c r="B64" t="s">
-        <v>250</v>
-      </c>
-      <c r="C64" t="s">
-        <v>251</v>
-      </c>
-      <c r="D64" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4">
-      <c r="A65" t="s">
-        <v>253</v>
-      </c>
-      <c r="B65" t="s">
-        <v>254</v>
-      </c>
-      <c r="C65" t="s">
-        <v>255</v>
-      </c>
-      <c r="D65" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4">
-      <c r="A66" t="s">
-        <v>257</v>
-      </c>
-      <c r="B66" t="s">
-        <v>258</v>
-      </c>
-      <c r="C66" t="s">
-        <v>259</v>
-      </c>
-      <c r="D66" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4">
-      <c r="A67" t="s">
-        <v>261</v>
-      </c>
-      <c r="B67" t="s">
-        <v>262</v>
-      </c>
-      <c r="C67" t="s">
-        <v>263</v>
-      </c>
-      <c r="D67" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4">
-      <c r="A68" t="s">
-        <v>265</v>
-      </c>
-      <c r="B68" t="s">
-        <v>266</v>
-      </c>
-      <c r="C68" t="s">
-        <v>267</v>
-      </c>
-      <c r="D68" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4">
-      <c r="A69" t="s">
-        <v>269</v>
-      </c>
-      <c r="B69" t="s">
-        <v>270</v>
-      </c>
-      <c r="C69" t="s">
-        <v>271</v>
-      </c>
-      <c r="D69" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4">
-      <c r="A70" t="s">
-        <v>273</v>
-      </c>
-      <c r="B70" t="s">
-        <v>274</v>
-      </c>
-      <c r="C70" t="s">
-        <v>275</v>
-      </c>
-      <c r="D70" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4">
-      <c r="A71" t="s">
-        <v>277</v>
-      </c>
-      <c r="B71" t="s">
-        <v>278</v>
-      </c>
-      <c r="C71" t="s">
-        <v>279</v>
-      </c>
-      <c r="D71" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4">
-      <c r="A72" t="s">
-        <v>281</v>
-      </c>
-      <c r="B72" t="s">
+      <c r="B76" t="s">
         <v>282</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C76" t="s">
         <v>283</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D76" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
-      <c r="A73" t="s">
+      <c r="E76" t="s">
         <v>285</v>
-      </c>
-      <c r="B73" t="s">
-        <v>286</v>
-      </c>
-      <c r="C73" t="s">
-        <v>287</v>
-      </c>
-      <c r="D73" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4">
-      <c r="C74" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4">
-      <c r="C75" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4">
-      <c r="C76" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4">
-      <c r="C77" t="s">
-        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -2818,239 +3030,251 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9878D5F-0194-4AC6-B566-F63E204E3C96}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.86328125" customWidth="1"/>
+    <col min="3" max="3" width="14.3984375" customWidth="1"/>
+    <col min="4" max="4" width="11.3984375" customWidth="1"/>
+    <col min="5" max="5" width="19.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D3" t="s">
+        <v>290</v>
+      </c>
+      <c r="E3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>291</v>
+      </c>
+      <c r="C4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E4" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>292</v>
+      </c>
+      <c r="C5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D5" t="s">
+        <v>292</v>
+      </c>
+      <c r="E5" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
         <v>293</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="C6" t="s">
+        <v>293</v>
+      </c>
+      <c r="D6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
         <v>294</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C7" t="s">
         <v>294</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D7" t="s">
         <v>294</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E7" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>295</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C8" t="s">
         <v>295</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D8" t="s">
         <v>295</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E8" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>296</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C9" t="s">
         <v>296</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D9" t="s">
         <v>296</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E9" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
         <v>297</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C10" t="s">
         <v>297</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D10" t="s">
         <v>297</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E10" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>298</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C11" t="s">
         <v>298</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D11" t="s">
         <v>298</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E11" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>299</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C12" t="s">
         <v>299</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D12" t="s">
         <v>299</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E12" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
         <v>300</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C13" t="s">
         <v>300</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D13" t="s">
         <v>300</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E13" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>454</v>
+      </c>
+      <c r="C14" t="s">
         <v>301</v>
       </c>
-      <c r="B9" t="s">
-        <v>301</v>
-      </c>
-      <c r="C9" t="s">
-        <v>301</v>
-      </c>
-      <c r="D9" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
-        <v>302</v>
-      </c>
-      <c r="B10" t="s">
-        <v>302</v>
-      </c>
-      <c r="C10" t="s">
-        <v>302</v>
-      </c>
-      <c r="D10" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+      <c r="D14" t="s">
+        <v>304</v>
+      </c>
+      <c r="E14" t="s">
         <v>303</v>
-      </c>
-      <c r="B11" t="s">
-        <v>303</v>
-      </c>
-      <c r="C11" t="s">
-        <v>303</v>
-      </c>
-      <c r="D11" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
-        <v>304</v>
-      </c>
-      <c r="B12" t="s">
-        <v>304</v>
-      </c>
-      <c r="C12" t="s">
-        <v>304</v>
-      </c>
-      <c r="D12" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
-        <v>305</v>
-      </c>
-      <c r="B13" t="s">
-        <v>305</v>
-      </c>
-      <c r="C13" t="s">
-        <v>305</v>
-      </c>
-      <c r="D13" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
-        <v>306</v>
-      </c>
-      <c r="B14" t="s">
-        <v>307</v>
-      </c>
-      <c r="C14" t="s">
-        <v>308</v>
-      </c>
-      <c r="D14" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="B15" t="s">
-        <v>309</v>
-      </c>
-      <c r="C15" t="s">
-        <v>309</v>
-      </c>
-      <c r="D15" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="B16" t="s">
-        <v>311</v>
-      </c>
-      <c r="C16" t="s">
-        <v>311</v>
-      </c>
-      <c r="D16" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="17" spans="3:4">
-      <c r="C17" t="s">
-        <v>313</v>
-      </c>
-      <c r="D17" t="s">
-        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -3060,94 +3284,118 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09178084-6EE9-4A4A-ACE4-85554F1DA5DB}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.59765625" customWidth="1"/>
+    <col min="4" max="4" width="17.86328125" customWidth="1"/>
+    <col min="5" max="5" width="20.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>293</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D2" t="s">
+        <v>308</v>
+      </c>
+      <c r="E2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D4" t="s">
+        <v>313</v>
+      </c>
+      <c r="E4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
         <v>315</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C5" t="s">
         <v>316</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D5" t="s">
         <v>317</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E5" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
         <v>320</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C7" t="s">
         <v>321</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E7" t="s">
         <v>322</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>323</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>324</v>
-      </c>
-      <c r="B5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C5" t="s">
-        <v>326</v>
-      </c>
-      <c r="D5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="D6" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>329</v>
-      </c>
-      <c r="B7" t="s">
-        <v>330</v>
-      </c>
-      <c r="D7" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -3158,15 +3406,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B779B73F-545A-4F4D-8CFE-66FFC11C3D0C}">
   <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
-    <col min="2" max="2" width="31.5703125" customWidth="1"/>
-    <col min="3" max="3" width="32.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.265625" customWidth="1"/>
+    <col min="2" max="2" width="31.59765625" customWidth="1"/>
+    <col min="3" max="3" width="32.1328125" customWidth="1"/>
     <col min="4" max="4" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3174,409 +3422,409 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C2" t="s">
+        <v>326</v>
+      </c>
+      <c r="D2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>328</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="C3" t="s">
+        <v>330</v>
+      </c>
+      <c r="D3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B4" t="s">
         <v>333</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C4" t="s">
         <v>334</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D4" t="s">
         <v>335</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="B5" t="s">
         <v>337</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C5" t="s">
         <v>338</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D5" t="s">
         <v>339</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="B6" t="s">
         <v>341</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C6" t="s">
         <v>342</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D6" t="s">
         <v>343</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
         <v>345</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C7" t="s">
         <v>346</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D7" t="s">
         <v>347</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="B8" t="s">
         <v>349</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C8" t="s">
         <v>350</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D8" t="s">
         <v>351</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D9" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
         <v>353</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B10" t="s">
         <v>354</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C10" t="s">
         <v>355</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D10" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
         <v>357</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B11" t="s">
         <v>358</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C11" t="s">
         <v>359</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D11" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="D9" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
+      <c r="B12" t="s">
         <v>362</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C12" t="s">
         <v>363</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D12" t="s">
         <v>364</v>
       </c>
-      <c r="D10" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+      <c r="B13" t="s">
         <v>366</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C13" t="s">
         <v>367</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D13" t="s">
         <v>368</v>
       </c>
-      <c r="D11" t="s">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+      <c r="B14" t="s">
         <v>370</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C14" t="s">
         <v>371</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D14" t="s">
         <v>372</v>
       </c>
-      <c r="D12" t="s">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
+      <c r="B15" t="s">
         <v>374</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C15" t="s">
         <v>375</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D15" t="s">
         <v>376</v>
       </c>
-      <c r="D13" t="s">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="B16" t="s">
         <v>378</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C16" t="s">
         <v>379</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D16" t="s">
         <v>380</v>
       </c>
-      <c r="D14" t="s">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+      <c r="B17" t="s">
         <v>382</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C17" t="s">
         <v>383</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D17" t="s">
         <v>384</v>
       </c>
-      <c r="D15" t="s">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
+      <c r="B18" t="s">
         <v>386</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C18" t="s">
         <v>387</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D18" t="s">
         <v>388</v>
       </c>
-      <c r="D16" t="s">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
+      <c r="B19" t="s">
         <v>390</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C19" t="s">
         <v>391</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D19" t="s">
         <v>392</v>
       </c>
-      <c r="D17" t="s">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
+      <c r="B20" t="s">
         <v>394</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C20" t="s">
         <v>395</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D20" t="s">
         <v>396</v>
       </c>
-      <c r="D18" t="s">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
+      <c r="B21" t="s">
         <v>398</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C21" t="s">
         <v>399</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D21" t="s">
         <v>400</v>
       </c>
-      <c r="D19" t="s">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
+      <c r="B22" t="s">
         <v>402</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C22" t="s">
         <v>403</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D22" t="s">
         <v>404</v>
       </c>
-      <c r="D20" t="s">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
         <v>406</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
         <v>407</v>
       </c>
-      <c r="C21" t="s">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B26" t="s">
         <v>408</v>
       </c>
-      <c r="D21" t="s">
+      <c r="C26" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
+      <c r="D26" t="s">
         <v>410</v>
       </c>
-      <c r="B22" t="s">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B27" t="s">
         <v>411</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C27" t="s">
         <v>412</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D27" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B28" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="C28" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="D28" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="B26" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B29" t="s">
         <v>417</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C29" t="s">
         <v>418</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D29" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="B27" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B30" t="s">
         <v>420</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C30" t="s">
         <v>421</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D30" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="B28" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B31" t="s">
         <v>423</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C31" t="s">
         <v>424</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D31" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="B29" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B32" t="s">
         <v>426</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C32" t="s">
         <v>427</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D32" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B33" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="B30" t="s">
+      <c r="C33" t="s">
         <v>429</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D33" t="s">
         <v>430</v>
       </c>
-      <c r="D30" t="s">
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B34" t="s">
         <v>431</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="B31" t="s">
+      <c r="C34" t="s">
         <v>432</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D34" t="s">
         <v>433</v>
-      </c>
-      <c r="D31" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="B32" t="s">
-        <v>435</v>
-      </c>
-      <c r="C32" t="s">
-        <v>436</v>
-      </c>
-      <c r="D32" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="33" spans="2:4">
-      <c r="B33" t="s">
-        <v>437</v>
-      </c>
-      <c r="C33" t="s">
-        <v>438</v>
-      </c>
-      <c r="D33" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4">
-      <c r="B34" t="s">
-        <v>440</v>
-      </c>
-      <c r="C34" t="s">
-        <v>441</v>
-      </c>
-      <c r="D34" t="s">
-        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -3587,9 +3835,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1661D22-A73B-4F85-82EE-7D613C5D43C3}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3597,107 +3845,107 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B2" t="s">
+        <v>435</v>
+      </c>
+      <c r="C2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D2" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B3" t="s">
+        <v>437</v>
+      </c>
+      <c r="C3" t="s">
+        <v>437</v>
+      </c>
+      <c r="D3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>440</v>
+      </c>
+      <c r="B5" t="s">
+        <v>440</v>
+      </c>
+      <c r="C5" t="s">
+        <v>440</v>
+      </c>
+      <c r="D5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>442</v>
+      </c>
+      <c r="B6" t="s">
+        <v>442</v>
+      </c>
+      <c r="C6" t="s">
+        <v>442</v>
+      </c>
+      <c r="D6" t="s">
         <v>443</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
         <v>444</v>
       </c>
-      <c r="C2" t="s">
-        <v>443</v>
-      </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>445</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="B8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C8" t="s">
+        <v>445</v>
+      </c>
+      <c r="D8" t="s">
         <v>446</v>
       </c>
-      <c r="B3" t="s">
-        <v>446</v>
-      </c>
-      <c r="C3" t="s">
-        <v>446</v>
-      </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="C9" t="s">
         <v>448</v>
-      </c>
-      <c r="B4" t="s">
-        <v>448</v>
-      </c>
-      <c r="C4" t="s">
-        <v>448</v>
-      </c>
-      <c r="D4" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>449</v>
-      </c>
-      <c r="B5" t="s">
-        <v>449</v>
-      </c>
-      <c r="C5" t="s">
-        <v>449</v>
-      </c>
-      <c r="D5" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>451</v>
-      </c>
-      <c r="B6" t="s">
-        <v>451</v>
-      </c>
-      <c r="C6" t="s">
-        <v>451</v>
-      </c>
-      <c r="D6" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="B7" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>454</v>
-      </c>
-      <c r="B8" t="s">
-        <v>454</v>
-      </c>
-      <c r="C8" t="s">
-        <v>454</v>
-      </c>
-      <c r="D8" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="B9" t="s">
-        <v>456</v>
-      </c>
-      <c r="C9" t="s">
-        <v>457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
production code and testing finished, last commit before moving to src
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/464195223dcae84f/Dokumente/OECD/RAnalysis/PRESS/data/keywords/review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="11_AD4DB114E441178AC67DF4704E97EB86683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CBB7C5F-5F72-43CB-82E7-D5742DE9605C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76FB9B2-4965-4EE3-8233-200B283408FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="2190" windowWidth="20145" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="457">
   <si>
     <t>en</t>
   </si>
@@ -46,9 +46,6 @@
     <t>fr</t>
   </si>
   <si>
-    <t xml:space="preserve">es </t>
-  </si>
-  <si>
     <t>de</t>
   </si>
   <si>
@@ -247,9 +244,6 @@
     <t>ciencia de los datos</t>
   </si>
   <si>
-    <t>Data Science</t>
-  </si>
-  <si>
     <t>data for development</t>
   </si>
   <si>
@@ -1403,6 +1397,18 @@
   </si>
   <si>
     <t>lfs</t>
+  </si>
+  <si>
+    <t>birth registr</t>
+  </si>
+  <si>
+    <t>civil registr</t>
+  </si>
+  <si>
+    <t>land registr</t>
+  </si>
+  <si>
+    <t>death registr</t>
   </si>
 </sst>
 </file>
@@ -1748,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="18.86328125" customWidth="1"/>
@@ -1759,7 +1765,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1768,10 +1774,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -1779,16 +1785,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -1796,16 +1802,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -1813,16 +1819,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>14</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -1830,16 +1836,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -1847,16 +1853,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -1864,16 +1870,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>26</v>
-      </c>
-      <c r="E7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -1881,16 +1887,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
-        <v>30</v>
-      </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -1898,16 +1904,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>32</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>33</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -1915,160 +1921,160 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
         <v>35</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>36</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>452</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>450</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>450</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>448</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>16</v>
       </c>
+      <c r="B19" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
       <c r="E19" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
@@ -2076,16 +2082,16 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" t="s">
         <v>70</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
         <v>71</v>
-      </c>
-      <c r="D20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
@@ -2093,16 +2099,16 @@
         <v>18</v>
       </c>
       <c r="B21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" t="s">
         <v>74</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>75</v>
-      </c>
-      <c r="D21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E21" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
@@ -2110,16 +2116,16 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" t="s">
         <v>78</v>
       </c>
-      <c r="C22" t="s">
+      <c r="E22" t="s">
         <v>79</v>
-      </c>
-      <c r="D22" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
@@ -2127,16 +2133,16 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" t="s">
         <v>82</v>
       </c>
-      <c r="C23" t="s">
+      <c r="E23" t="s">
         <v>83</v>
-      </c>
-      <c r="D23" t="s">
-        <v>84</v>
-      </c>
-      <c r="E23" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -2144,16 +2150,16 @@
         <v>21</v>
       </c>
       <c r="B24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" t="s">
         <v>86</v>
       </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>87</v>
-      </c>
-      <c r="D24" t="s">
-        <v>88</v>
-      </c>
-      <c r="E24" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -2161,16 +2167,16 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" t="s">
         <v>90</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25" t="s">
         <v>91</v>
-      </c>
-      <c r="D25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E25" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
@@ -2178,16 +2184,16 @@
         <v>23</v>
       </c>
       <c r="B26" t="s">
+        <v>92</v>
+      </c>
+      <c r="C26" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" t="s">
         <v>94</v>
       </c>
-      <c r="C26" t="s">
+      <c r="E26" t="s">
         <v>95</v>
-      </c>
-      <c r="D26" t="s">
-        <v>96</v>
-      </c>
-      <c r="E26" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
@@ -2195,16 +2201,16 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" t="s">
         <v>98</v>
-      </c>
-      <c r="C27" t="s">
-        <v>98</v>
-      </c>
-      <c r="D27" t="s">
-        <v>99</v>
-      </c>
-      <c r="E27" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
@@ -2212,16 +2218,16 @@
         <v>25</v>
       </c>
       <c r="B28" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" t="s">
         <v>101</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E28" t="s">
         <v>102</v>
-      </c>
-      <c r="D28" t="s">
-        <v>103</v>
-      </c>
-      <c r="E28" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
@@ -2229,16 +2235,16 @@
         <v>26</v>
       </c>
       <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" t="s">
         <v>105</v>
       </c>
-      <c r="C29" t="s">
+      <c r="E29" t="s">
         <v>106</v>
-      </c>
-      <c r="D29" t="s">
-        <v>107</v>
-      </c>
-      <c r="E29" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -2246,16 +2252,16 @@
         <v>27</v>
       </c>
       <c r="B30" t="s">
+        <v>107</v>
+      </c>
+      <c r="C30" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" t="s">
         <v>109</v>
       </c>
-      <c r="C30" t="s">
+      <c r="E30" t="s">
         <v>110</v>
-      </c>
-      <c r="D30" t="s">
-        <v>111</v>
-      </c>
-      <c r="E30" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
@@ -2263,16 +2269,16 @@
         <v>28</v>
       </c>
       <c r="B31" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" t="s">
+        <v>112</v>
+      </c>
+      <c r="D31" t="s">
         <v>113</v>
       </c>
-      <c r="C31" t="s">
+      <c r="E31" t="s">
         <v>114</v>
-      </c>
-      <c r="D31" t="s">
-        <v>115</v>
-      </c>
-      <c r="E31" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
@@ -2280,16 +2286,16 @@
         <v>29</v>
       </c>
       <c r="B32" t="s">
+        <v>115</v>
+      </c>
+      <c r="C32" t="s">
+        <v>116</v>
+      </c>
+      <c r="D32" t="s">
         <v>117</v>
       </c>
-      <c r="C32" t="s">
+      <c r="E32" t="s">
         <v>118</v>
-      </c>
-      <c r="D32" t="s">
-        <v>119</v>
-      </c>
-      <c r="E32" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
@@ -2297,16 +2303,16 @@
         <v>30</v>
       </c>
       <c r="B33" t="s">
+        <v>119</v>
+      </c>
+      <c r="C33" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" t="s">
         <v>121</v>
       </c>
-      <c r="C33" t="s">
+      <c r="E33" t="s">
         <v>122</v>
-      </c>
-      <c r="D33" t="s">
-        <v>123</v>
-      </c>
-      <c r="E33" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
@@ -2314,16 +2320,16 @@
         <v>31</v>
       </c>
       <c r="B34" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" t="s">
+        <v>124</v>
+      </c>
+      <c r="D34" t="s">
         <v>125</v>
       </c>
-      <c r="C34" t="s">
+      <c r="E34" t="s">
         <v>126</v>
-      </c>
-      <c r="D34" t="s">
-        <v>127</v>
-      </c>
-      <c r="E34" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
@@ -2331,16 +2337,16 @@
         <v>32</v>
       </c>
       <c r="B35" t="s">
+        <v>127</v>
+      </c>
+      <c r="C35" t="s">
+        <v>128</v>
+      </c>
+      <c r="D35" t="s">
         <v>129</v>
       </c>
-      <c r="C35" t="s">
+      <c r="E35" t="s">
         <v>130</v>
-      </c>
-      <c r="D35" t="s">
-        <v>131</v>
-      </c>
-      <c r="E35" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
@@ -2348,16 +2354,16 @@
         <v>33</v>
       </c>
       <c r="B36" t="s">
+        <v>131</v>
+      </c>
+      <c r="C36" t="s">
+        <v>132</v>
+      </c>
+      <c r="D36" t="s">
         <v>133</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" t="s">
         <v>134</v>
-      </c>
-      <c r="D36" t="s">
-        <v>135</v>
-      </c>
-      <c r="E36" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.45">
@@ -2365,16 +2371,16 @@
         <v>34</v>
       </c>
       <c r="B37" t="s">
+        <v>135</v>
+      </c>
+      <c r="C37" t="s">
+        <v>136</v>
+      </c>
+      <c r="D37" t="s">
         <v>137</v>
       </c>
-      <c r="C37" t="s">
+      <c r="E37" t="s">
         <v>138</v>
-      </c>
-      <c r="D37" t="s">
-        <v>139</v>
-      </c>
-      <c r="E37" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
@@ -2382,16 +2388,16 @@
         <v>35</v>
       </c>
       <c r="B38" t="s">
+        <v>139</v>
+      </c>
+      <c r="C38" t="s">
+        <v>140</v>
+      </c>
+      <c r="D38" t="s">
         <v>141</v>
       </c>
-      <c r="C38" t="s">
+      <c r="E38" t="s">
         <v>142</v>
-      </c>
-      <c r="D38" t="s">
-        <v>143</v>
-      </c>
-      <c r="E38" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
@@ -2399,16 +2405,16 @@
         <v>36</v>
       </c>
       <c r="B39" t="s">
+        <v>143</v>
+      </c>
+      <c r="C39" t="s">
+        <v>144</v>
+      </c>
+      <c r="D39" t="s">
         <v>145</v>
       </c>
-      <c r="C39" t="s">
+      <c r="E39" t="s">
         <v>146</v>
-      </c>
-      <c r="D39" t="s">
-        <v>147</v>
-      </c>
-      <c r="E39" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
@@ -2416,16 +2422,16 @@
         <v>37</v>
       </c>
       <c r="B40" t="s">
+        <v>147</v>
+      </c>
+      <c r="C40" t="s">
+        <v>148</v>
+      </c>
+      <c r="D40" t="s">
         <v>149</v>
       </c>
-      <c r="C40" t="s">
+      <c r="E40" t="s">
         <v>150</v>
-      </c>
-      <c r="D40" t="s">
-        <v>151</v>
-      </c>
-      <c r="E40" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.45">
@@ -2433,7 +2439,7 @@
         <v>37</v>
       </c>
       <c r="D41" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
@@ -2441,16 +2447,16 @@
         <v>38</v>
       </c>
       <c r="B42" t="s">
+        <v>151</v>
+      </c>
+      <c r="C42" t="s">
+        <v>152</v>
+      </c>
+      <c r="D42" t="s">
         <v>153</v>
       </c>
-      <c r="C42" t="s">
+      <c r="E42" t="s">
         <v>154</v>
-      </c>
-      <c r="D42" t="s">
-        <v>155</v>
-      </c>
-      <c r="E42" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
@@ -2458,7 +2464,7 @@
         <v>38</v>
       </c>
       <c r="D43" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
@@ -2466,16 +2472,16 @@
         <v>39</v>
       </c>
       <c r="B44" t="s">
+        <v>155</v>
+      </c>
+      <c r="C44" t="s">
+        <v>156</v>
+      </c>
+      <c r="D44" t="s">
         <v>157</v>
       </c>
-      <c r="C44" t="s">
+      <c r="E44" t="s">
         <v>158</v>
-      </c>
-      <c r="D44" t="s">
-        <v>159</v>
-      </c>
-      <c r="E44" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
@@ -2483,16 +2489,16 @@
         <v>40</v>
       </c>
       <c r="B45" t="s">
+        <v>159</v>
+      </c>
+      <c r="C45" t="s">
+        <v>160</v>
+      </c>
+      <c r="D45" t="s">
         <v>161</v>
       </c>
-      <c r="C45" t="s">
+      <c r="E45" t="s">
         <v>162</v>
-      </c>
-      <c r="D45" t="s">
-        <v>163</v>
-      </c>
-      <c r="E45" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
@@ -2500,16 +2506,16 @@
         <v>41</v>
       </c>
       <c r="B46" t="s">
+        <v>163</v>
+      </c>
+      <c r="C46" t="s">
+        <v>164</v>
+      </c>
+      <c r="D46" t="s">
         <v>165</v>
       </c>
-      <c r="C46" t="s">
+      <c r="E46" t="s">
         <v>166</v>
-      </c>
-      <c r="D46" t="s">
-        <v>167</v>
-      </c>
-      <c r="E46" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
@@ -2517,16 +2523,16 @@
         <v>42</v>
       </c>
       <c r="B47" t="s">
+        <v>167</v>
+      </c>
+      <c r="C47" t="s">
+        <v>168</v>
+      </c>
+      <c r="D47" t="s">
         <v>169</v>
       </c>
-      <c r="C47" t="s">
+      <c r="E47" t="s">
         <v>170</v>
-      </c>
-      <c r="D47" t="s">
-        <v>171</v>
-      </c>
-      <c r="E47" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
@@ -2534,16 +2540,16 @@
         <v>43</v>
       </c>
       <c r="B48" t="s">
+        <v>171</v>
+      </c>
+      <c r="C48" t="s">
+        <v>172</v>
+      </c>
+      <c r="D48" t="s">
         <v>173</v>
       </c>
-      <c r="C48" t="s">
+      <c r="E48" t="s">
         <v>174</v>
-      </c>
-      <c r="D48" t="s">
-        <v>175</v>
-      </c>
-      <c r="E48" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.45">
@@ -2551,16 +2557,16 @@
         <v>44</v>
       </c>
       <c r="B49" t="s">
+        <v>175</v>
+      </c>
+      <c r="C49" t="s">
+        <v>176</v>
+      </c>
+      <c r="D49" t="s">
         <v>177</v>
       </c>
-      <c r="C49" t="s">
+      <c r="E49" t="s">
         <v>178</v>
-      </c>
-      <c r="D49" t="s">
-        <v>179</v>
-      </c>
-      <c r="E49" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.45">
@@ -2568,16 +2574,16 @@
         <v>45</v>
       </c>
       <c r="B50" t="s">
+        <v>179</v>
+      </c>
+      <c r="C50" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" t="s">
         <v>181</v>
       </c>
-      <c r="C50" t="s">
+      <c r="E50" t="s">
         <v>182</v>
-      </c>
-      <c r="D50" t="s">
-        <v>183</v>
-      </c>
-      <c r="E50" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.45">
@@ -2585,16 +2591,16 @@
         <v>46</v>
       </c>
       <c r="B51" t="s">
+        <v>183</v>
+      </c>
+      <c r="C51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D51" t="s">
         <v>185</v>
       </c>
-      <c r="C51" t="s">
+      <c r="E51" t="s">
         <v>186</v>
-      </c>
-      <c r="D51" t="s">
-        <v>187</v>
-      </c>
-      <c r="E51" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.45">
@@ -2602,16 +2608,16 @@
         <v>47</v>
       </c>
       <c r="B52" t="s">
+        <v>187</v>
+      </c>
+      <c r="C52" t="s">
+        <v>188</v>
+      </c>
+      <c r="D52" t="s">
         <v>189</v>
       </c>
-      <c r="C52" t="s">
+      <c r="E52" t="s">
         <v>190</v>
-      </c>
-      <c r="D52" t="s">
-        <v>191</v>
-      </c>
-      <c r="E52" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.45">
@@ -2619,16 +2625,16 @@
         <v>48</v>
       </c>
       <c r="B53" t="s">
+        <v>191</v>
+      </c>
+      <c r="C53" t="s">
+        <v>192</v>
+      </c>
+      <c r="D53" t="s">
         <v>193</v>
       </c>
-      <c r="C53" t="s">
+      <c r="E53" t="s">
         <v>194</v>
-      </c>
-      <c r="D53" t="s">
-        <v>195</v>
-      </c>
-      <c r="E53" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.45">
@@ -2636,16 +2642,16 @@
         <v>49</v>
       </c>
       <c r="B54" t="s">
+        <v>195</v>
+      </c>
+      <c r="C54" t="s">
+        <v>196</v>
+      </c>
+      <c r="D54" t="s">
         <v>197</v>
       </c>
-      <c r="C54" t="s">
+      <c r="E54" t="s">
         <v>198</v>
-      </c>
-      <c r="D54" t="s">
-        <v>199</v>
-      </c>
-      <c r="E54" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.45">
@@ -2653,16 +2659,16 @@
         <v>50</v>
       </c>
       <c r="B55" t="s">
+        <v>199</v>
+      </c>
+      <c r="C55" t="s">
+        <v>188</v>
+      </c>
+      <c r="D55" t="s">
+        <v>200</v>
+      </c>
+      <c r="E55" t="s">
         <v>201</v>
-      </c>
-      <c r="C55" t="s">
-        <v>190</v>
-      </c>
-      <c r="D55" t="s">
-        <v>202</v>
-      </c>
-      <c r="E55" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.45">
@@ -2670,16 +2676,16 @@
         <v>51</v>
       </c>
       <c r="B56" t="s">
+        <v>202</v>
+      </c>
+      <c r="C56" t="s">
+        <v>192</v>
+      </c>
+      <c r="D56" t="s">
+        <v>203</v>
+      </c>
+      <c r="E56" t="s">
         <v>204</v>
-      </c>
-      <c r="C56" t="s">
-        <v>194</v>
-      </c>
-      <c r="D56" t="s">
-        <v>205</v>
-      </c>
-      <c r="E56" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.45">
@@ -2687,16 +2693,16 @@
         <v>52</v>
       </c>
       <c r="B57" t="s">
+        <v>205</v>
+      </c>
+      <c r="C57" t="s">
+        <v>206</v>
+      </c>
+      <c r="D57" t="s">
         <v>207</v>
       </c>
-      <c r="C57" t="s">
+      <c r="E57" t="s">
         <v>208</v>
-      </c>
-      <c r="D57" t="s">
-        <v>209</v>
-      </c>
-      <c r="E57" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.45">
@@ -2704,16 +2710,16 @@
         <v>53</v>
       </c>
       <c r="B58" t="s">
+        <v>209</v>
+      </c>
+      <c r="C58" t="s">
+        <v>210</v>
+      </c>
+      <c r="D58" t="s">
         <v>211</v>
       </c>
-      <c r="C58" t="s">
+      <c r="E58" t="s">
         <v>212</v>
-      </c>
-      <c r="D58" t="s">
-        <v>213</v>
-      </c>
-      <c r="E58" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.45">
@@ -2721,16 +2727,16 @@
         <v>54</v>
       </c>
       <c r="B59" t="s">
+        <v>213</v>
+      </c>
+      <c r="C59" t="s">
+        <v>214</v>
+      </c>
+      <c r="D59" t="s">
         <v>215</v>
       </c>
-      <c r="C59" t="s">
+      <c r="E59" t="s">
         <v>216</v>
-      </c>
-      <c r="D59" t="s">
-        <v>217</v>
-      </c>
-      <c r="E59" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.45">
@@ -2738,16 +2744,16 @@
         <v>55</v>
       </c>
       <c r="B60" t="s">
+        <v>217</v>
+      </c>
+      <c r="C60" t="s">
+        <v>218</v>
+      </c>
+      <c r="D60" t="s">
         <v>219</v>
       </c>
-      <c r="C60" t="s">
+      <c r="E60" t="s">
         <v>220</v>
-      </c>
-      <c r="D60" t="s">
-        <v>221</v>
-      </c>
-      <c r="E60" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.45">
@@ -2755,16 +2761,16 @@
         <v>56</v>
       </c>
       <c r="B61" t="s">
+        <v>221</v>
+      </c>
+      <c r="C61" t="s">
+        <v>222</v>
+      </c>
+      <c r="D61" t="s">
         <v>223</v>
       </c>
-      <c r="C61" t="s">
+      <c r="E61" t="s">
         <v>224</v>
-      </c>
-      <c r="D61" t="s">
-        <v>225</v>
-      </c>
-      <c r="E61" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.45">
@@ -2772,16 +2778,16 @@
         <v>57</v>
       </c>
       <c r="B62" t="s">
+        <v>225</v>
+      </c>
+      <c r="C62" t="s">
+        <v>226</v>
+      </c>
+      <c r="D62" t="s">
         <v>227</v>
       </c>
-      <c r="C62" t="s">
+      <c r="E62" t="s">
         <v>228</v>
-      </c>
-      <c r="D62" t="s">
-        <v>229</v>
-      </c>
-      <c r="E62" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.45">
@@ -2789,16 +2795,16 @@
         <v>58</v>
       </c>
       <c r="B63" t="s">
+        <v>229</v>
+      </c>
+      <c r="C63" t="s">
+        <v>230</v>
+      </c>
+      <c r="D63" t="s">
         <v>231</v>
       </c>
-      <c r="C63" t="s">
+      <c r="E63" t="s">
         <v>232</v>
-      </c>
-      <c r="D63" t="s">
-        <v>233</v>
-      </c>
-      <c r="E63" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.45">
@@ -2806,16 +2812,16 @@
         <v>59</v>
       </c>
       <c r="B64" t="s">
+        <v>233</v>
+      </c>
+      <c r="C64" t="s">
+        <v>234</v>
+      </c>
+      <c r="D64" t="s">
         <v>235</v>
       </c>
-      <c r="C64" t="s">
+      <c r="E64" t="s">
         <v>236</v>
-      </c>
-      <c r="D64" t="s">
-        <v>237</v>
-      </c>
-      <c r="E64" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.45">
@@ -2823,16 +2829,16 @@
         <v>60</v>
       </c>
       <c r="B65" t="s">
+        <v>237</v>
+      </c>
+      <c r="C65" t="s">
+        <v>238</v>
+      </c>
+      <c r="D65" t="s">
         <v>239</v>
       </c>
-      <c r="C65" t="s">
+      <c r="E65" t="s">
         <v>240</v>
-      </c>
-      <c r="D65" t="s">
-        <v>241</v>
-      </c>
-      <c r="E65" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.45">
@@ -2840,16 +2846,16 @@
         <v>61</v>
       </c>
       <c r="B66" t="s">
+        <v>241</v>
+      </c>
+      <c r="C66" t="s">
+        <v>242</v>
+      </c>
+      <c r="D66" t="s">
         <v>243</v>
       </c>
-      <c r="C66" t="s">
+      <c r="E66" t="s">
         <v>244</v>
-      </c>
-      <c r="D66" t="s">
-        <v>245</v>
-      </c>
-      <c r="E66" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.45">
@@ -2857,16 +2863,16 @@
         <v>62</v>
       </c>
       <c r="B67" t="s">
+        <v>245</v>
+      </c>
+      <c r="C67" t="s">
+        <v>246</v>
+      </c>
+      <c r="D67" t="s">
         <v>247</v>
       </c>
-      <c r="C67" t="s">
+      <c r="E67" t="s">
         <v>248</v>
-      </c>
-      <c r="D67" t="s">
-        <v>249</v>
-      </c>
-      <c r="E67" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.45">
@@ -2874,16 +2880,16 @@
         <v>63</v>
       </c>
       <c r="B68" t="s">
+        <v>249</v>
+      </c>
+      <c r="C68" t="s">
+        <v>250</v>
+      </c>
+      <c r="D68" t="s">
         <v>251</v>
       </c>
-      <c r="C68" t="s">
+      <c r="E68" t="s">
         <v>252</v>
-      </c>
-      <c r="D68" t="s">
-        <v>253</v>
-      </c>
-      <c r="E68" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.45">
@@ -2891,16 +2897,16 @@
         <v>64</v>
       </c>
       <c r="B69" t="s">
+        <v>253</v>
+      </c>
+      <c r="C69" t="s">
+        <v>254</v>
+      </c>
+      <c r="D69" t="s">
         <v>255</v>
       </c>
-      <c r="C69" t="s">
+      <c r="E69" t="s">
         <v>256</v>
-      </c>
-      <c r="D69" t="s">
-        <v>257</v>
-      </c>
-      <c r="E69" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.45">
@@ -2908,16 +2914,16 @@
         <v>65</v>
       </c>
       <c r="B70" t="s">
+        <v>257</v>
+      </c>
+      <c r="C70" t="s">
+        <v>262</v>
+      </c>
+      <c r="D70" t="s">
         <v>259</v>
       </c>
-      <c r="C70" t="s">
-        <v>264</v>
-      </c>
-      <c r="D70" t="s">
-        <v>261</v>
-      </c>
       <c r="E70" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
@@ -2925,16 +2931,16 @@
         <v>66</v>
       </c>
       <c r="B71" t="s">
+        <v>261</v>
+      </c>
+      <c r="C71" t="s">
+        <v>258</v>
+      </c>
+      <c r="D71" t="s">
         <v>263</v>
       </c>
-      <c r="C71" t="s">
-        <v>260</v>
-      </c>
-      <c r="D71" t="s">
-        <v>265</v>
-      </c>
       <c r="E71" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.45">
@@ -2942,16 +2948,16 @@
         <v>67</v>
       </c>
       <c r="B72" t="s">
+        <v>265</v>
+      </c>
+      <c r="C72" t="s">
+        <v>266</v>
+      </c>
+      <c r="D72" t="s">
         <v>267</v>
       </c>
-      <c r="C72" t="s">
+      <c r="E72" t="s">
         <v>268</v>
-      </c>
-      <c r="D72" t="s">
-        <v>269</v>
-      </c>
-      <c r="E72" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.45">
@@ -2959,16 +2965,16 @@
         <v>68</v>
       </c>
       <c r="B73" t="s">
+        <v>269</v>
+      </c>
+      <c r="C73" t="s">
+        <v>270</v>
+      </c>
+      <c r="D73" t="s">
         <v>271</v>
       </c>
-      <c r="C73" t="s">
+      <c r="E73" t="s">
         <v>272</v>
-      </c>
-      <c r="D73" t="s">
-        <v>273</v>
-      </c>
-      <c r="E73" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.45">
@@ -2976,16 +2982,16 @@
         <v>69</v>
       </c>
       <c r="B74" t="s">
+        <v>273</v>
+      </c>
+      <c r="C74" t="s">
+        <v>274</v>
+      </c>
+      <c r="D74" t="s">
         <v>275</v>
       </c>
-      <c r="C74" t="s">
+      <c r="E74" t="s">
         <v>276</v>
-      </c>
-      <c r="D74" t="s">
-        <v>277</v>
-      </c>
-      <c r="E74" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.45">
@@ -2993,16 +2999,16 @@
         <v>70</v>
       </c>
       <c r="B75" t="s">
+        <v>277</v>
+      </c>
+      <c r="C75" t="s">
+        <v>278</v>
+      </c>
+      <c r="D75" t="s">
         <v>279</v>
       </c>
-      <c r="C75" t="s">
-        <v>280</v>
-      </c>
-      <c r="D75" t="s">
-        <v>281</v>
-      </c>
       <c r="E75" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.45">
@@ -3010,16 +3016,48 @@
         <v>71</v>
       </c>
       <c r="B76" t="s">
+        <v>280</v>
+      </c>
+      <c r="C76" t="s">
+        <v>281</v>
+      </c>
+      <c r="D76" t="s">
         <v>282</v>
       </c>
-      <c r="C76" t="s">
+      <c r="E76" t="s">
         <v>283</v>
       </c>
-      <c r="D76" t="s">
-        <v>284</v>
-      </c>
-      <c r="E76" t="s">
-        <v>285</v>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A77">
+        <v>72</v>
+      </c>
+      <c r="B77" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A78">
+        <v>73</v>
+      </c>
+      <c r="B78" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A79">
+        <v>74</v>
+      </c>
+      <c r="B79" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A80">
+        <v>75</v>
+      </c>
+      <c r="B80" t="s">
+        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -3041,7 +3079,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3050,10 +3088,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -3061,16 +3099,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -3078,16 +3116,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="E3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -3095,16 +3133,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="D4" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -3112,16 +3150,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -3129,16 +3167,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -3146,16 +3184,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="D7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -3163,16 +3201,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E8" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -3180,16 +3218,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C9" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D9" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E9" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -3197,16 +3235,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="D10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -3214,16 +3252,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -3231,16 +3269,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E12" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -3248,16 +3286,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="D13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -3265,16 +3303,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C14" t="s">
+        <v>299</v>
+      </c>
+      <c r="D14" t="s">
+        <v>302</v>
+      </c>
+      <c r="E14" t="s">
         <v>301</v>
-      </c>
-      <c r="D14" t="s">
-        <v>304</v>
-      </c>
-      <c r="E14" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -3294,7 +3332,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3303,10 +3341,10 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -3314,16 +3352,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D2" t="s">
         <v>306</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>307</v>
-      </c>
-      <c r="D2" t="s">
-        <v>308</v>
-      </c>
-      <c r="E2" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -3331,7 +3369,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -3339,16 +3377,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" t="s">
+        <v>310</v>
+      </c>
+      <c r="D4" t="s">
         <v>311</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>312</v>
-      </c>
-      <c r="D4" t="s">
-        <v>313</v>
-      </c>
-      <c r="E4" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -3356,16 +3394,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>313</v>
+      </c>
+      <c r="C5" t="s">
+        <v>314</v>
+      </c>
+      <c r="D5" t="s">
         <v>315</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>316</v>
-      </c>
-      <c r="D5" t="s">
-        <v>317</v>
-      </c>
-      <c r="E5" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -3373,7 +3411,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -3381,13 +3419,13 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
+        <v>318</v>
+      </c>
+      <c r="C7" t="s">
+        <v>319</v>
+      </c>
+      <c r="E7" t="s">
         <v>320</v>
-      </c>
-      <c r="C7" t="s">
-        <v>321</v>
-      </c>
-      <c r="E7" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -3395,7 +3433,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -3422,409 +3460,409 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C2" t="s">
         <v>324</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>325</v>
-      </c>
-      <c r="C2" t="s">
-        <v>326</v>
-      </c>
-      <c r="D2" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C3" t="s">
         <v>328</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" t="s">
         <v>329</v>
-      </c>
-      <c r="C3" t="s">
-        <v>330</v>
-      </c>
-      <c r="D3" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>330</v>
+      </c>
+      <c r="B4" t="s">
+        <v>331</v>
+      </c>
+      <c r="C4" t="s">
         <v>332</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>333</v>
-      </c>
-      <c r="C4" t="s">
-        <v>334</v>
-      </c>
-      <c r="D4" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>334</v>
+      </c>
+      <c r="B5" t="s">
+        <v>335</v>
+      </c>
+      <c r="C5" t="s">
         <v>336</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>337</v>
-      </c>
-      <c r="C5" t="s">
-        <v>338</v>
-      </c>
-      <c r="D5" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B6" t="s">
+        <v>339</v>
+      </c>
+      <c r="C6" t="s">
         <v>340</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>341</v>
-      </c>
-      <c r="C6" t="s">
-        <v>342</v>
-      </c>
-      <c r="D6" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B7" t="s">
+        <v>343</v>
+      </c>
+      <c r="C7" t="s">
         <v>344</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>345</v>
-      </c>
-      <c r="C7" t="s">
-        <v>346</v>
-      </c>
-      <c r="D7" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B8" t="s">
+        <v>347</v>
+      </c>
+      <c r="C8" t="s">
         <v>348</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>349</v>
-      </c>
-      <c r="C8" t="s">
-        <v>350</v>
-      </c>
-      <c r="D8" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D9" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>351</v>
+      </c>
+      <c r="B10" t="s">
+        <v>352</v>
+      </c>
+      <c r="C10" t="s">
         <v>353</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
         <v>354</v>
-      </c>
-      <c r="C10" t="s">
-        <v>355</v>
-      </c>
-      <c r="D10" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>355</v>
+      </c>
+      <c r="B11" t="s">
+        <v>356</v>
+      </c>
+      <c r="C11" t="s">
         <v>357</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>358</v>
-      </c>
-      <c r="C11" t="s">
-        <v>359</v>
-      </c>
-      <c r="D11" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>359</v>
+      </c>
+      <c r="B12" t="s">
+        <v>360</v>
+      </c>
+      <c r="C12" t="s">
         <v>361</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>362</v>
-      </c>
-      <c r="C12" t="s">
-        <v>363</v>
-      </c>
-      <c r="D12" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>363</v>
+      </c>
+      <c r="B13" t="s">
+        <v>364</v>
+      </c>
+      <c r="C13" t="s">
         <v>365</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
         <v>366</v>
-      </c>
-      <c r="C13" t="s">
-        <v>367</v>
-      </c>
-      <c r="D13" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
+        <v>367</v>
+      </c>
+      <c r="B14" t="s">
+        <v>368</v>
+      </c>
+      <c r="C14" t="s">
         <v>369</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>370</v>
-      </c>
-      <c r="C14" t="s">
-        <v>371</v>
-      </c>
-      <c r="D14" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
+        <v>371</v>
+      </c>
+      <c r="B15" t="s">
+        <v>372</v>
+      </c>
+      <c r="C15" t="s">
         <v>373</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>374</v>
-      </c>
-      <c r="C15" t="s">
-        <v>375</v>
-      </c>
-      <c r="D15" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
+        <v>375</v>
+      </c>
+      <c r="B16" t="s">
+        <v>376</v>
+      </c>
+      <c r="C16" t="s">
         <v>377</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>378</v>
-      </c>
-      <c r="C16" t="s">
-        <v>379</v>
-      </c>
-      <c r="D16" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>379</v>
+      </c>
+      <c r="B17" t="s">
+        <v>380</v>
+      </c>
+      <c r="C17" t="s">
         <v>381</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
         <v>382</v>
-      </c>
-      <c r="C17" t="s">
-        <v>383</v>
-      </c>
-      <c r="D17" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B18" t="s">
+        <v>384</v>
+      </c>
+      <c r="C18" t="s">
         <v>385</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>386</v>
-      </c>
-      <c r="C18" t="s">
-        <v>387</v>
-      </c>
-      <c r="D18" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
+        <v>387</v>
+      </c>
+      <c r="B19" t="s">
+        <v>388</v>
+      </c>
+      <c r="C19" t="s">
         <v>389</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>390</v>
-      </c>
-      <c r="C19" t="s">
-        <v>391</v>
-      </c>
-      <c r="D19" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
+        <v>391</v>
+      </c>
+      <c r="B20" t="s">
+        <v>392</v>
+      </c>
+      <c r="C20" t="s">
         <v>393</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>394</v>
-      </c>
-      <c r="C20" t="s">
-        <v>395</v>
-      </c>
-      <c r="D20" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
+        <v>395</v>
+      </c>
+      <c r="B21" t="s">
+        <v>396</v>
+      </c>
+      <c r="C21" t="s">
         <v>397</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>398</v>
-      </c>
-      <c r="C21" t="s">
-        <v>399</v>
-      </c>
-      <c r="D21" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
+        <v>399</v>
+      </c>
+      <c r="B22" t="s">
+        <v>400</v>
+      </c>
+      <c r="C22" t="s">
         <v>401</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
         <v>402</v>
-      </c>
-      <c r="C22" t="s">
-        <v>403</v>
-      </c>
-      <c r="D22" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
+        <v>406</v>
+      </c>
+      <c r="C26" t="s">
+        <v>407</v>
+      </c>
+      <c r="D26" t="s">
         <v>408</v>
-      </c>
-      <c r="C26" t="s">
-        <v>409</v>
-      </c>
-      <c r="D26" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
+        <v>409</v>
+      </c>
+      <c r="C27" t="s">
+        <v>410</v>
+      </c>
+      <c r="D27" t="s">
         <v>411</v>
-      </c>
-      <c r="C27" t="s">
-        <v>412</v>
-      </c>
-      <c r="D27" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
+        <v>412</v>
+      </c>
+      <c r="C28" t="s">
+        <v>413</v>
+      </c>
+      <c r="D28" t="s">
         <v>414</v>
-      </c>
-      <c r="C28" t="s">
-        <v>415</v>
-      </c>
-      <c r="D28" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
+        <v>415</v>
+      </c>
+      <c r="C29" t="s">
+        <v>416</v>
+      </c>
+      <c r="D29" t="s">
         <v>417</v>
-      </c>
-      <c r="C29" t="s">
-        <v>418</v>
-      </c>
-      <c r="D29" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
+        <v>418</v>
+      </c>
+      <c r="C30" t="s">
+        <v>419</v>
+      </c>
+      <c r="D30" t="s">
         <v>420</v>
-      </c>
-      <c r="C30" t="s">
-        <v>421</v>
-      </c>
-      <c r="D30" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
+        <v>421</v>
+      </c>
+      <c r="C31" t="s">
+        <v>422</v>
+      </c>
+      <c r="D31" t="s">
         <v>423</v>
-      </c>
-      <c r="C31" t="s">
-        <v>424</v>
-      </c>
-      <c r="D31" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C32" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D32" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
+        <v>426</v>
+      </c>
+      <c r="C33" t="s">
+        <v>427</v>
+      </c>
+      <c r="D33" t="s">
         <v>428</v>
-      </c>
-      <c r="C33" t="s">
-        <v>429</v>
-      </c>
-      <c r="D33" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
+        <v>429</v>
+      </c>
+      <c r="C34" t="s">
+        <v>430</v>
+      </c>
+      <c r="D34" t="s">
         <v>431</v>
-      </c>
-      <c r="C34" t="s">
-        <v>432</v>
-      </c>
-      <c r="D34" t="s">
-        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -3845,107 +3883,107 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D2" t="s">
         <v>434</v>
-      </c>
-      <c r="B2" t="s">
-        <v>435</v>
-      </c>
-      <c r="C2" t="s">
-        <v>434</v>
-      </c>
-      <c r="D2" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D3" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="B4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="C4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D5" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B6" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="C6" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D6" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C8" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="D8" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C9" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated keywords (AI -> statistics), creation of final markers
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/464195223dcae84f/Dokumente/OECD/RAnalysis/PRESS/data/keywords/review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9A756046-C61B-4D94-9F3B-EB36523D8CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6C89D91-0834-4F7B-8F2B-67B6F765EED7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EC8464-8B5C-4562-B991-9EB6DCBF4276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1837" yWindow="1837" windowWidth="20146" windowHeight="13756" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
     <sheet name="statistics acronyms" sheetId="2" r:id="rId2"/>
     <sheet name="stat blacklist" sheetId="6" r:id="rId3"/>
-    <sheet name="AI" sheetId="7" r:id="rId4"/>
-    <sheet name="AI acronyms" sheetId="8" r:id="rId5"/>
+    <sheet name="AI acronyms" sheetId="8" r:id="rId4"/>
+    <sheet name="AI" sheetId="7" r:id="rId5"/>
     <sheet name="gender" sheetId="3" r:id="rId6"/>
     <sheet name="gender acronyms" sheetId="4" r:id="rId7"/>
   </sheets>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="609">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="616">
   <si>
     <t>id</t>
   </si>
@@ -1860,20 +1860,41 @@
     <t>fgm</t>
   </si>
   <si>
-    <t>MG</t>
-  </si>
-  <si>
     <t>SDSR</t>
   </si>
   <si>
     <t>Hochzeit</t>
+  </si>
+  <si>
+    <t>quantum computing</t>
+  </si>
+  <si>
+    <t>calcul quantique</t>
+  </si>
+  <si>
+    <t>computación cuántica</t>
+  </si>
+  <si>
+    <t>Quantencomputing</t>
+  </si>
+  <si>
+    <t>generative AI</t>
+  </si>
+  <si>
+    <t>IA générative</t>
+  </si>
+  <si>
+    <t>IA generativa</t>
+  </si>
+  <si>
+    <t>generative KI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1936,6 +1957,26 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF375623"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF375623"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1958,7 +1999,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1972,6 +2013,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2253,7 +2300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="24.1328125" customWidth="1"/>
@@ -3740,11 +3787,255 @@
         <v>338</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45"/>
-    <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45"/>
-    <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45"/>
-    <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45"/>
-    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45"/>
+    <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A89" s="9">
+        <v>85</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="E89" s="11" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A90" s="9">
+        <v>86</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="E90" s="10" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A91" s="9">
+        <v>87</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="E91" s="10" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A92" s="9">
+        <v>88</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E92" s="10" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A93" s="9">
+        <v>88</v>
+      </c>
+      <c r="B93" s="3"/>
+      <c r="C93" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="D93" s="3"/>
+      <c r="E93" s="10"/>
+    </row>
+    <row r="94" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A94" s="9">
+        <v>89</v>
+      </c>
+      <c r="B94" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="C94" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="D94" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="E94" s="9" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A95" s="9">
+        <v>90</v>
+      </c>
+      <c r="B95" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="C95" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="E95" s="9" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A96" s="9">
+        <v>91</v>
+      </c>
+      <c r="B96" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="C96" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="D96" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A97" s="9">
+        <v>92</v>
+      </c>
+      <c r="B97" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="C97" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="D97" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A98" s="9">
+        <v>93</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="E98" s="10" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A99" s="9">
+        <v>94</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="C99" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="D99" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A100" s="9">
+        <v>95</v>
+      </c>
+      <c r="B100" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C100" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="D100" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A101" s="9">
+        <v>96</v>
+      </c>
+      <c r="B101" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="C101" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="D101" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A102" s="9">
+        <v>97</v>
+      </c>
+      <c r="B102" s="9" t="s">
+        <v>608</v>
+      </c>
+      <c r="C102" s="9" t="s">
+        <v>609</v>
+      </c>
+      <c r="D102" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A103" s="9">
+        <v>98</v>
+      </c>
+      <c r="B103" s="9" t="s">
+        <v>612</v>
+      </c>
+      <c r="C103" s="9" t="s">
+        <v>613</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>614</v>
+      </c>
+      <c r="E103" s="9" t="s">
+        <v>615</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3898,7 +4189,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4034,9 +4325,45 @@
         <v>369</v>
       </c>
     </row>
-    <row r="17" x14ac:dyDescent="0.45"/>
-    <row r="18" x14ac:dyDescent="0.45"/>
-    <row r="19" x14ac:dyDescent="0.45"/>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A17" s="9">
+        <v>15</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18" s="9">
+        <v>16</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>463</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="9">
+        <v>17</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4176,6 +4503,98 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A530C6-6E1E-4869-A1CA-FDC34F8192D0}">
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>465</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6AF1E86-DE73-4CDF-BE84-D18DA4C485BA}">
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4501,98 +4920,6 @@
       </c>
       <c r="E19" t="s">
         <v>456</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34A530C6-6E1E-4869-A1CA-FDC34F8192D0}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>460</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -4710,7 +5037,7 @@
         <v>484</v>
       </c>
       <c r="E6" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5162,7 +5489,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1661D22-A73B-4F85-82EE-7D613C5D43C3}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
@@ -5261,7 +5588,7 @@
         <v>601</v>
       </c>
       <c r="D6" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="E6" t="s">
         <v>602</v>
@@ -5282,17 +5609,6 @@
       </c>
       <c r="E7" t="s">
         <v>605</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>606</v>
-      </c>
-      <c r="D8" t="s">
-        <v>607</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
processing after entire crs stat predicted by adding add info (RegionName, DonorType, iso, FS, SIDS)
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EC8464-8B5C-4562-B991-9EB6DCBF4276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A00FE2A-30F4-400C-8B32-B68B7C8F3A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="615">
   <si>
     <t>id</t>
   </si>
@@ -1144,9 +1144,6 @@
   </si>
   <si>
     <t>INE</t>
-  </si>
-  <si>
-    <t>NSA</t>
   </si>
   <si>
     <t>NSS</t>
@@ -3792,16 +3789,16 @@
         <v>85</v>
       </c>
       <c r="B89" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C89" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="D89" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="D89" s="3" t="s">
+      <c r="E89" s="11" t="s">
         <v>396</v>
-      </c>
-      <c r="E89" s="11" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3809,16 +3806,16 @@
         <v>86</v>
       </c>
       <c r="B90" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C90" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="D90" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="E90" s="10" t="s">
         <v>400</v>
-      </c>
-      <c r="E90" s="10" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3826,16 +3823,16 @@
         <v>87</v>
       </c>
       <c r="B91" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C91" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="D91" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="D91" s="3" t="s">
+      <c r="E91" s="10" t="s">
         <v>404</v>
-      </c>
-      <c r="E91" s="10" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3843,16 +3840,16 @@
         <v>88</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C92" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="D92" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="E92" s="10" t="s">
         <v>408</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3861,7 +3858,7 @@
       </c>
       <c r="B93" s="3"/>
       <c r="C93" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="10"/>
@@ -3874,10 +3871,10 @@
         <v>329</v>
       </c>
       <c r="C94" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="D94" s="9" t="s">
         <v>411</v>
-      </c>
-      <c r="D94" s="9" t="s">
-        <v>412</v>
       </c>
       <c r="E94" s="9" t="s">
         <v>330</v>
@@ -3888,16 +3885,16 @@
         <v>90</v>
       </c>
       <c r="B95" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="C95" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="D95" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="C95" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="D95" s="9" t="s">
+      <c r="E95" s="9" t="s">
         <v>414</v>
-      </c>
-      <c r="E95" s="9" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3905,16 +3902,16 @@
         <v>91</v>
       </c>
       <c r="B96" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="C96" s="9" t="s">
         <v>423</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="D96" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="D96" s="9" t="s">
+      <c r="E96" s="9" t="s">
         <v>425</v>
-      </c>
-      <c r="E96" s="9" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3922,16 +3919,16 @@
         <v>92</v>
       </c>
       <c r="B97" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="C97" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="D97" s="9" t="s">
         <v>428</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="E97" s="9" t="s">
         <v>429</v>
-      </c>
-      <c r="E97" s="9" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3939,16 +3936,16 @@
         <v>93</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="C98" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="C98" s="3" t="s">
+      <c r="D98" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="D98" s="3" t="s">
+      <c r="E98" s="10" t="s">
         <v>433</v>
-      </c>
-      <c r="E98" s="10" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3956,16 +3953,16 @@
         <v>94</v>
       </c>
       <c r="B99" s="9" t="s">
+        <v>434</v>
+      </c>
+      <c r="C99" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="D99" s="9" t="s">
         <v>436</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="E99" s="9" t="s">
         <v>437</v>
-      </c>
-      <c r="E99" s="9" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3973,16 +3970,16 @@
         <v>95</v>
       </c>
       <c r="B100" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="C100" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="D100" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="E100" s="9" t="s">
         <v>441</v>
-      </c>
-      <c r="E100" s="9" t="s">
-        <v>442</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -3990,16 +3987,16 @@
         <v>96</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C101" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="D101" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="E101" s="9" t="s">
         <v>447</v>
-      </c>
-      <c r="D101" s="9" t="s">
-        <v>400</v>
-      </c>
-      <c r="E101" s="9" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4007,16 +4004,16 @@
         <v>97</v>
       </c>
       <c r="B102" s="9" t="s">
+        <v>607</v>
+      </c>
+      <c r="C102" s="9" t="s">
         <v>608</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="D102" s="9" t="s">
         <v>609</v>
       </c>
-      <c r="D102" s="9" t="s">
+      <c r="E102" s="9" t="s">
         <v>610</v>
-      </c>
-      <c r="E102" s="9" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4024,16 +4021,16 @@
         <v>98</v>
       </c>
       <c r="B103" s="9" t="s">
+        <v>611</v>
+      </c>
+      <c r="C103" s="9" t="s">
         <v>612</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="D103" s="12" t="s">
         <v>613</v>
       </c>
-      <c r="D103" s="12" t="s">
+      <c r="E103" s="9" t="s">
         <v>614</v>
-      </c>
-      <c r="E103" s="9" t="s">
-        <v>615</v>
       </c>
     </row>
   </sheetData>
@@ -4304,25 +4301,23 @@
       <c r="D15" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>368</v>
-      </c>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>371</v>
-      </c>
       <c r="E16" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -4330,16 +4325,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>461</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -4347,7 +4342,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
@@ -4358,7 +4353,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
@@ -4401,16 +4396,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C2" t="s">
         <v>372</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>373</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>374</v>
-      </c>
-      <c r="E2" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4418,7 +4413,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4426,16 +4421,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C4" t="s">
         <v>377</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>378</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>379</v>
-      </c>
-      <c r="E4" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4443,16 +4438,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>380</v>
+      </c>
+      <c r="C5" t="s">
         <v>381</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>382</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>383</v>
-      </c>
-      <c r="E5" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4460,7 +4455,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4468,16 +4463,16 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>385</v>
+      </c>
+      <c r="C7" t="s">
         <v>386</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>387</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>388</v>
-      </c>
-      <c r="E7" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4485,16 +4480,16 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
+        <v>389</v>
+      </c>
+      <c r="C8" t="s">
         <v>390</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>391</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>392</v>
-      </c>
-      <c r="E8" t="s">
-        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -4529,7 +4524,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4537,7 +4532,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4545,7 +4540,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4553,16 +4548,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>459</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>461</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4570,7 +4565,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4578,7 +4573,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4586,7 +4581,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
   </sheetData>
@@ -4627,16 +4622,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>396</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4644,16 +4639,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>400</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4661,16 +4656,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>404</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4678,16 +4673,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="6" t="s">
         <v>408</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4696,7 +4691,7 @@
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="6"/>
@@ -4709,10 +4704,10 @@
         <v>329</v>
       </c>
       <c r="C7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D7" t="s">
         <v>411</v>
-      </c>
-      <c r="D7" t="s">
-        <v>412</v>
       </c>
       <c r="E7" t="s">
         <v>330</v>
@@ -4723,16 +4718,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
+        <v>412</v>
+      </c>
+      <c r="C8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D8" t="s">
         <v>413</v>
       </c>
-      <c r="C8" t="s">
-        <v>413</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>414</v>
-      </c>
-      <c r="E8" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -4740,16 +4735,16 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>415</v>
+      </c>
+      <c r="C9" t="s">
         <v>416</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>417</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>418</v>
-      </c>
-      <c r="E9" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -4757,16 +4752,16 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
+        <v>419</v>
+      </c>
+      <c r="C10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D10" t="s">
         <v>420</v>
       </c>
-      <c r="C10" t="s">
-        <v>420</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>421</v>
-      </c>
-      <c r="E10" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -4774,16 +4769,16 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
+        <v>422</v>
+      </c>
+      <c r="C11" t="s">
         <v>423</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>424</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>425</v>
-      </c>
-      <c r="E11" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4791,16 +4786,16 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
+        <v>426</v>
+      </c>
+      <c r="C12" t="s">
         <v>427</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>428</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>429</v>
-      </c>
-      <c r="E12" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -4808,16 +4803,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="6" t="s">
         <v>433</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -4825,16 +4820,16 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
+        <v>434</v>
+      </c>
+      <c r="C14" t="s">
         <v>435</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>436</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>437</v>
-      </c>
-      <c r="E14" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -4842,16 +4837,16 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
+        <v>438</v>
+      </c>
+      <c r="C15" t="s">
         <v>439</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>440</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>441</v>
-      </c>
-      <c r="E15" t="s">
-        <v>442</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -4859,16 +4854,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
+        <v>442</v>
+      </c>
+      <c r="C16" t="s">
         <v>443</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>444</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>445</v>
-      </c>
-      <c r="E16" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -4876,16 +4871,16 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C17" t="s">
+        <v>446</v>
+      </c>
+      <c r="D17" t="s">
+        <v>399</v>
+      </c>
+      <c r="E17" t="s">
         <v>447</v>
-      </c>
-      <c r="D17" t="s">
-        <v>400</v>
-      </c>
-      <c r="E17" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -4893,16 +4888,16 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
+        <v>448</v>
+      </c>
+      <c r="C18" t="s">
         <v>449</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>450</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>451</v>
-      </c>
-      <c r="E18" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -4910,16 +4905,16 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
+        <v>452</v>
+      </c>
+      <c r="C19" t="s">
         <v>453</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>454</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>455</v>
-      </c>
-      <c r="E19" t="s">
-        <v>456</v>
       </c>
     </row>
   </sheetData>
@@ -4960,16 +4955,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>465</v>
+      </c>
+      <c r="C2" t="s">
         <v>466</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>467</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>468</v>
-      </c>
-      <c r="E2" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4977,16 +4972,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>469</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" t="s">
         <v>471</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>472</v>
-      </c>
-      <c r="E3" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4994,16 +4989,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>473</v>
+      </c>
+      <c r="C4" t="s">
         <v>474</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>475</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>476</v>
-      </c>
-      <c r="E4" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5011,16 +5006,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>477</v>
+      </c>
+      <c r="C5" t="s">
         <v>478</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>479</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>480</v>
-      </c>
-      <c r="E5" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5028,16 +5023,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>481</v>
+      </c>
+      <c r="C6" t="s">
         <v>482</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>483</v>
       </c>
-      <c r="D6" t="s">
-        <v>484</v>
-      </c>
       <c r="E6" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5045,16 +5040,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>484</v>
+      </c>
+      <c r="C7" t="s">
         <v>485</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>486</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>487</v>
-      </c>
-      <c r="E7" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -5062,16 +5057,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>488</v>
+      </c>
+      <c r="C8" t="s">
         <v>489</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>490</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>491</v>
-      </c>
-      <c r="E8" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -5079,16 +5074,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>492</v>
+      </c>
+      <c r="C9" t="s">
         <v>493</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>494</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>495</v>
-      </c>
-      <c r="E9" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -5096,16 +5091,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>496</v>
+      </c>
+      <c r="C10" t="s">
         <v>497</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>498</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>499</v>
-      </c>
-      <c r="E10" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -5113,16 +5108,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>500</v>
+      </c>
+      <c r="C11" t="s">
         <v>501</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>502</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>503</v>
-      </c>
-      <c r="E11" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -5130,16 +5125,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>504</v>
+      </c>
+      <c r="C12" t="s">
         <v>505</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>506</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>507</v>
-      </c>
-      <c r="E12" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -5147,16 +5142,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>508</v>
+      </c>
+      <c r="C13" t="s">
         <v>509</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>510</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>511</v>
-      </c>
-      <c r="E13" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -5164,16 +5159,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>512</v>
+      </c>
+      <c r="C14" t="s">
         <v>513</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>514</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>515</v>
-      </c>
-      <c r="E14" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -5181,16 +5176,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
+        <v>516</v>
+      </c>
+      <c r="C15" t="s">
         <v>517</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>518</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>519</v>
-      </c>
-      <c r="E15" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -5198,16 +5193,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
+        <v>520</v>
+      </c>
+      <c r="C16" t="s">
         <v>521</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>522</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>523</v>
-      </c>
-      <c r="E16" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -5215,16 +5210,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
+        <v>524</v>
+      </c>
+      <c r="C17" t="s">
         <v>525</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>526</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>527</v>
-      </c>
-      <c r="E17" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -5232,16 +5227,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
+        <v>528</v>
+      </c>
+      <c r="C18" t="s">
         <v>529</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>530</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>531</v>
-      </c>
-      <c r="E18" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -5249,16 +5244,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
+        <v>532</v>
+      </c>
+      <c r="C19" t="s">
         <v>533</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>534</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>535</v>
-      </c>
-      <c r="E19" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
@@ -5266,16 +5261,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
+        <v>536</v>
+      </c>
+      <c r="C20" t="s">
         <v>537</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>538</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>539</v>
-      </c>
-      <c r="E20" t="s">
-        <v>540</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
@@ -5283,16 +5278,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>540</v>
+      </c>
+      <c r="C21" t="s">
         <v>541</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>542</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>543</v>
-      </c>
-      <c r="E21" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
@@ -5300,16 +5295,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>544</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>546</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" t="s">
         <v>547</v>
-      </c>
-      <c r="E22" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
@@ -5317,16 +5312,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
+        <v>548</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>549</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>550</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" t="s">
         <v>551</v>
-      </c>
-      <c r="E23" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -5334,16 +5329,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
+        <v>552</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>554</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="E24" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -5351,16 +5346,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>554</v>
+      </c>
+      <c r="C25" t="s">
         <v>555</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>556</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>557</v>
-      </c>
-      <c r="E25" t="s">
-        <v>558</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
@@ -5368,16 +5363,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
+        <v>558</v>
+      </c>
+      <c r="C26" t="s">
         <v>559</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>560</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>561</v>
-      </c>
-      <c r="E26" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
@@ -5385,16 +5380,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
+        <v>562</v>
+      </c>
+      <c r="C27" t="s">
         <v>563</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>564</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>565</v>
-      </c>
-      <c r="E27" t="s">
-        <v>566</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
@@ -5402,16 +5397,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
+        <v>566</v>
+      </c>
+      <c r="C28" t="s">
         <v>567</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>568</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>569</v>
-      </c>
-      <c r="E28" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
@@ -5419,16 +5414,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
+        <v>570</v>
+      </c>
+      <c r="C29" t="s">
         <v>571</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>572</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>573</v>
-      </c>
-      <c r="E29" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -5436,16 +5431,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
+        <v>574</v>
+      </c>
+      <c r="C30" t="s">
         <v>575</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>576</v>
       </c>
-      <c r="D30" t="s">
-        <v>577</v>
-      </c>
       <c r="E30" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
@@ -5453,16 +5448,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
+        <v>577</v>
+      </c>
+      <c r="C31" t="s">
         <v>578</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>579</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>580</v>
-      </c>
-      <c r="E31" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
@@ -5470,16 +5465,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
+        <v>581</v>
+      </c>
+      <c r="C32" t="s">
         <v>582</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>583</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>584</v>
-      </c>
-      <c r="E32" t="s">
-        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -5514,16 +5509,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C2" t="s">
         <v>586</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E2" t="s">
         <v>587</v>
-      </c>
-      <c r="D2" t="s">
-        <v>587</v>
-      </c>
-      <c r="E2" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -5531,16 +5526,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>588</v>
+      </c>
+      <c r="C3" t="s">
         <v>589</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>590</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>591</v>
-      </c>
-      <c r="E3" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -5548,16 +5543,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>592</v>
+      </c>
+      <c r="C4" t="s">
         <v>593</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>594</v>
       </c>
-      <c r="D4" t="s">
-        <v>595</v>
-      </c>
       <c r="E4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5565,16 +5560,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>595</v>
+      </c>
+      <c r="C5" t="s">
         <v>596</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>597</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>598</v>
-      </c>
-      <c r="E5" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5582,16 +5577,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>599</v>
+      </c>
+      <c r="C6" t="s">
         <v>600</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>605</v>
+      </c>
+      <c r="E6" t="s">
         <v>601</v>
-      </c>
-      <c r="D6" t="s">
-        <v>606</v>
-      </c>
-      <c r="E6" t="s">
-        <v>602</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5599,16 +5594,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>602</v>
+      </c>
+      <c r="C7" t="s">
         <v>603</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>603</v>
+      </c>
+      <c r="E7" t="s">
         <v>604</v>
-      </c>
-      <c r="D7" t="s">
-        <v>604</v>
-      </c>
-      <c r="E7" t="s">
-        <v>605</v>
       </c>
     </row>
   </sheetData>
@@ -5628,6 +5623,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -5888,15 +5892,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
   <ds:schemaRefs>
@@ -5909,6 +5904,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5925,12 +5928,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated final press pipeline, output, keyword adjustments
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A00FE2A-30F4-400C-8B32-B68B7C8F3A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D05AEC-E955-4F41-AD84-8F72D54AC743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="623">
   <si>
     <t>id</t>
   </si>
@@ -1089,9 +1089,6 @@
     <t>gpsdd</t>
   </si>
   <si>
-    <t>odw</t>
-  </si>
-  <si>
     <t>data4sdg</t>
   </si>
   <si>
@@ -1885,6 +1882,33 @@
   </si>
   <si>
     <t>generative KI</t>
+  </si>
+  <si>
+    <t>birth registration</t>
+  </si>
+  <si>
+    <t>civil registration</t>
+  </si>
+  <si>
+    <t>land registration</t>
+  </si>
+  <si>
+    <t>business registration</t>
+  </si>
+  <si>
+    <t>civil registry</t>
+  </si>
+  <si>
+    <t>land registry</t>
+  </si>
+  <si>
+    <t>birth registry</t>
+  </si>
+  <si>
+    <t>business registry</t>
+  </si>
+  <si>
+    <t>death registration</t>
   </si>
 </sst>
 </file>
@@ -2297,7 +2321,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="24.1328125" customWidth="1"/>
@@ -2430,7 +2454,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>615</v>
       </c>
       <c r="C8" t="s">
         <v>29</v>
@@ -2444,1593 +2468,1682 @@
     </row>
     <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>35</v>
-      </c>
+        <v>618</v>
+      </c>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" t="s">
-        <v>47</v>
+        <v>619</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" t="s">
-        <v>51</v>
+        <v>616</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>55</v>
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A17">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A18">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A19">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" t="s">
-        <v>75</v>
+        <v>620</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A20">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" t="s">
-        <v>79</v>
+        <v>614</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A21">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>82</v>
-      </c>
-      <c r="E21" t="s">
-        <v>83</v>
+        <v>54</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A22">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E22" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A23">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>91</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A24">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B24" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="C24" t="s">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>94</v>
+        <v>66</v>
       </c>
       <c r="E24" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A25">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="E25" t="s">
-        <v>99</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A26">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="E26" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A27">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="D27" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="E27" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A28">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B28" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
-        <v>109</v>
+        <v>82</v>
       </c>
       <c r="E28" t="s">
-        <v>110</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A29">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="D29" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="E29" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A30">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="C30" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="D30" t="s">
-        <v>117</v>
+        <v>90</v>
       </c>
       <c r="E30" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A31">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B31" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="D31" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="E31" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A32">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="D32" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A33">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="D33" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="E33" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A34">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="D34" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="E34" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A35">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="C35" t="s">
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="D35" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="E35" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A36">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B36" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="C36" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="D36" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
       <c r="E36" t="s">
-        <v>142</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A37">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B37" t="s">
-        <v>143</v>
+        <v>115</v>
       </c>
       <c r="C37" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="D37" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
       <c r="E37" t="s">
-        <v>146</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A38">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B38" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="C38" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
       <c r="D38" t="s">
-        <v>149</v>
+        <v>121</v>
       </c>
       <c r="E38" t="s">
-        <v>150</v>
+        <v>122</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A39">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="C39" t="s">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="D39" t="s">
-        <v>153</v>
+        <v>125</v>
       </c>
       <c r="E39" t="s">
-        <v>154</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A40">
-        <v>37</v>
+        <v>31</v>
+      </c>
+      <c r="B40" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" t="s">
+        <v>128</v>
       </c>
       <c r="D40" t="s">
-        <v>155</v>
+        <v>129</v>
+      </c>
+      <c r="E40" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A41">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B41" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="C41" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="D41" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="E41" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A42">
-        <v>38</v>
-      </c>
-      <c r="D42" t="s">
-        <v>160</v>
+        <v>32</v>
+      </c>
+      <c r="B42" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A43">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B43" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C43" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
       <c r="D43" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="E43" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A44">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="C44" t="s">
-        <v>166</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="E44" t="s">
-        <v>168</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A45">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>169</v>
+        <v>143</v>
       </c>
       <c r="C45" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="E45" t="s">
-        <v>172</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A46">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B46" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="C46" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="D46" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="E46" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A47">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B47" t="s">
-        <v>177</v>
+        <v>151</v>
       </c>
       <c r="C47" t="s">
-        <v>178</v>
+        <v>152</v>
       </c>
       <c r="D47" t="s">
-        <v>179</v>
+        <v>153</v>
       </c>
       <c r="E47" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A48">
-        <v>44</v>
-      </c>
-      <c r="B48" t="s">
-        <v>181</v>
-      </c>
-      <c r="C48" t="s">
-        <v>182</v>
+        <v>37</v>
       </c>
       <c r="D48" t="s">
-        <v>183</v>
-      </c>
-      <c r="E48" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A49">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B49" t="s">
-        <v>185</v>
+        <v>156</v>
       </c>
       <c r="C49" t="s">
-        <v>186</v>
+        <v>157</v>
       </c>
       <c r="D49" t="s">
-        <v>187</v>
+        <v>158</v>
       </c>
       <c r="E49" t="s">
-        <v>188</v>
+        <v>159</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A50">
-        <v>46</v>
-      </c>
-      <c r="B50" t="s">
-        <v>189</v>
-      </c>
-      <c r="C50" t="s">
-        <v>190</v>
+        <v>38</v>
       </c>
       <c r="D50" t="s">
-        <v>191</v>
-      </c>
-      <c r="E50" t="s">
-        <v>192</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A51">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B51" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
       <c r="C51" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="D51" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
       <c r="E51" t="s">
-        <v>196</v>
+        <v>164</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A52">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B52" t="s">
-        <v>197</v>
+        <v>165</v>
       </c>
       <c r="C52" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="D52" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
       <c r="E52" t="s">
-        <v>200</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A53">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B53" t="s">
-        <v>201</v>
+        <v>169</v>
       </c>
       <c r="C53" t="s">
-        <v>202</v>
+        <v>170</v>
       </c>
       <c r="D53" t="s">
-        <v>203</v>
+        <v>171</v>
       </c>
       <c r="E53" t="s">
-        <v>204</v>
+        <v>172</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A54">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B54" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
       <c r="C54" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
       <c r="D54" t="s">
-        <v>206</v>
+        <v>175</v>
       </c>
       <c r="E54" t="s">
-        <v>207</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A55">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B55" t="s">
-        <v>208</v>
+        <v>177</v>
       </c>
       <c r="C55" t="s">
-        <v>198</v>
+        <v>178</v>
       </c>
       <c r="D55" t="s">
-        <v>209</v>
+        <v>179</v>
       </c>
       <c r="E55" t="s">
-        <v>210</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A56">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="B56" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
       <c r="C56" t="s">
-        <v>212</v>
+        <v>182</v>
       </c>
       <c r="D56" t="s">
-        <v>213</v>
+        <v>183</v>
       </c>
       <c r="E56" t="s">
-        <v>214</v>
+        <v>184</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A57">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B57" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
       <c r="C57" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
       <c r="D57" t="s">
-        <v>217</v>
+        <v>187</v>
       </c>
       <c r="E57" t="s">
-        <v>218</v>
+        <v>188</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A58">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B58" t="s">
-        <v>219</v>
+        <v>189</v>
       </c>
       <c r="C58" t="s">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="D58" t="s">
-        <v>221</v>
+        <v>191</v>
       </c>
       <c r="E58" t="s">
-        <v>222</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A59">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B59" t="s">
-        <v>223</v>
+        <v>193</v>
       </c>
       <c r="C59" t="s">
-        <v>224</v>
+        <v>194</v>
       </c>
       <c r="D59" t="s">
-        <v>225</v>
+        <v>195</v>
       </c>
       <c r="E59" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A60">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B60" t="s">
-        <v>227</v>
+        <v>197</v>
       </c>
       <c r="C60" t="s">
-        <v>228</v>
+        <v>198</v>
       </c>
       <c r="D60" t="s">
-        <v>229</v>
+        <v>199</v>
       </c>
       <c r="E60" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A61">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B61" t="s">
-        <v>231</v>
+        <v>201</v>
       </c>
       <c r="C61" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
       <c r="D61" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
       <c r="E61" t="s">
-        <v>234</v>
+        <v>204</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A62">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B62" t="s">
-        <v>235</v>
+        <v>205</v>
       </c>
       <c r="C62" t="s">
-        <v>236</v>
+        <v>194</v>
       </c>
       <c r="D62" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
       <c r="E62" t="s">
-        <v>238</v>
+        <v>207</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A63">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B63" t="s">
-        <v>239</v>
+        <v>208</v>
       </c>
       <c r="C63" t="s">
-        <v>240</v>
+        <v>198</v>
       </c>
       <c r="D63" t="s">
-        <v>241</v>
+        <v>209</v>
       </c>
       <c r="E63" t="s">
-        <v>242</v>
+        <v>210</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A64">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B64" t="s">
-        <v>243</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>244</v>
+        <v>212</v>
       </c>
       <c r="D64" t="s">
-        <v>245</v>
+        <v>213</v>
       </c>
       <c r="E64" t="s">
-        <v>246</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A65">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B65" t="s">
-        <v>247</v>
+        <v>215</v>
       </c>
       <c r="C65" t="s">
-        <v>248</v>
+        <v>216</v>
       </c>
       <c r="D65" t="s">
-        <v>249</v>
+        <v>217</v>
       </c>
       <c r="E65" t="s">
-        <v>250</v>
+        <v>218</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A66">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B66" t="s">
-        <v>251</v>
+        <v>219</v>
       </c>
       <c r="C66" t="s">
-        <v>252</v>
+        <v>220</v>
       </c>
       <c r="D66" t="s">
-        <v>253</v>
+        <v>221</v>
       </c>
       <c r="E66" t="s">
-        <v>254</v>
+        <v>222</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A67">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B67" t="s">
-        <v>255</v>
+        <v>223</v>
       </c>
       <c r="C67" t="s">
-        <v>256</v>
+        <v>224</v>
       </c>
       <c r="D67" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="E67" t="s">
-        <v>258</v>
+        <v>226</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A68">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B68" t="s">
-        <v>259</v>
+        <v>227</v>
       </c>
       <c r="C68" t="s">
-        <v>260</v>
+        <v>228</v>
       </c>
       <c r="D68" t="s">
-        <v>261</v>
+        <v>229</v>
       </c>
       <c r="E68" t="s">
-        <v>262</v>
+        <v>230</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A69">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B69" t="s">
-        <v>263</v>
+        <v>231</v>
       </c>
       <c r="C69" t="s">
-        <v>264</v>
+        <v>232</v>
       </c>
       <c r="D69" t="s">
-        <v>265</v>
+        <v>233</v>
       </c>
       <c r="E69" t="s">
-        <v>266</v>
+        <v>234</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A70">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B70" t="s">
-        <v>267</v>
+        <v>235</v>
       </c>
       <c r="C70" t="s">
-        <v>268</v>
+        <v>236</v>
       </c>
       <c r="D70" t="s">
-        <v>269</v>
+        <v>237</v>
       </c>
       <c r="E70" t="s">
-        <v>270</v>
+        <v>238</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A71">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B71" t="s">
-        <v>271</v>
+        <v>239</v>
       </c>
       <c r="C71" t="s">
-        <v>272</v>
+        <v>240</v>
       </c>
       <c r="D71" t="s">
-        <v>273</v>
+        <v>241</v>
       </c>
       <c r="E71" t="s">
-        <v>274</v>
+        <v>242</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A72">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B72" t="s">
-        <v>275</v>
+        <v>243</v>
       </c>
       <c r="C72" t="s">
-        <v>276</v>
+        <v>244</v>
       </c>
       <c r="D72" t="s">
-        <v>277</v>
+        <v>245</v>
       </c>
       <c r="E72" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A73">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B73" t="s">
-        <v>279</v>
+        <v>247</v>
       </c>
       <c r="C73" t="s">
-        <v>280</v>
+        <v>248</v>
       </c>
       <c r="D73" t="s">
-        <v>281</v>
+        <v>249</v>
       </c>
       <c r="E73" t="s">
-        <v>282</v>
+        <v>250</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A74">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B74" t="s">
-        <v>283</v>
+        <v>251</v>
       </c>
       <c r="C74" t="s">
-        <v>284</v>
+        <v>252</v>
       </c>
       <c r="D74" t="s">
-        <v>285</v>
+        <v>253</v>
       </c>
       <c r="E74" t="s">
-        <v>286</v>
+        <v>254</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A75">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B75" t="s">
-        <v>287</v>
+        <v>255</v>
       </c>
       <c r="C75" t="s">
-        <v>288</v>
+        <v>256</v>
       </c>
       <c r="D75" t="s">
-        <v>289</v>
+        <v>257</v>
       </c>
       <c r="E75" t="s">
-        <v>290</v>
+        <v>258</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A76">
-        <v>72</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>294</v>
+        <v>64</v>
+      </c>
+      <c r="B76" t="s">
+        <v>259</v>
+      </c>
+      <c r="C76" t="s">
+        <v>260</v>
+      </c>
+      <c r="D76" t="s">
+        <v>261</v>
+      </c>
+      <c r="E76" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A77">
-        <v>73</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>298</v>
+        <v>65</v>
+      </c>
+      <c r="B77" t="s">
+        <v>263</v>
+      </c>
+      <c r="C77" t="s">
+        <v>264</v>
+      </c>
+      <c r="D77" t="s">
+        <v>265</v>
+      </c>
+      <c r="E77" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A78">
-        <v>74</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+        <v>66</v>
+      </c>
+      <c r="B78" t="s">
+        <v>267</v>
+      </c>
+      <c r="C78" t="s">
+        <v>268</v>
+      </c>
+      <c r="D78" t="s">
+        <v>269</v>
+      </c>
+      <c r="E78" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A79">
-        <v>75</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>303</v>
+        <v>67</v>
+      </c>
+      <c r="B79" t="s">
+        <v>271</v>
+      </c>
+      <c r="C79" t="s">
+        <v>272</v>
+      </c>
+      <c r="D79" t="s">
+        <v>273</v>
+      </c>
+      <c r="E79" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A80">
-        <v>76</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>309</v>
+        <v>68</v>
+      </c>
+      <c r="B80" t="s">
+        <v>275</v>
+      </c>
+      <c r="C80" t="s">
+        <v>276</v>
+      </c>
+      <c r="D80" t="s">
+        <v>277</v>
+      </c>
+      <c r="E80" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A81">
-        <v>77</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="E81" s="6" t="s">
-        <v>313</v>
+        <v>69</v>
+      </c>
+      <c r="B81" t="s">
+        <v>279</v>
+      </c>
+      <c r="C81" t="s">
+        <v>280</v>
+      </c>
+      <c r="D81" t="s">
+        <v>281</v>
+      </c>
+      <c r="E81" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A82">
-        <v>78</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>316</v>
+        <v>70</v>
+      </c>
+      <c r="B82" t="s">
+        <v>283</v>
+      </c>
+      <c r="C82" t="s">
+        <v>284</v>
+      </c>
+      <c r="D82" t="s">
+        <v>285</v>
+      </c>
+      <c r="E82" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A83">
-        <v>79</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="C83" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="E83" s="6" t="s">
-        <v>320</v>
+        <v>71</v>
+      </c>
+      <c r="B83" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A84">
-        <v>80</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E84" s="6" t="s">
-        <v>324</v>
+        <v>71</v>
+      </c>
+      <c r="B84" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A85">
-        <v>81</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="E85" s="6" t="s">
-        <v>328</v>
+        <v>71</v>
+      </c>
+      <c r="B85" t="s">
+        <v>617</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A86">
-        <v>82</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="E86" s="6" t="s">
-        <v>330</v>
+        <v>72</v>
+      </c>
+      <c r="B86" t="s">
+        <v>287</v>
+      </c>
+      <c r="C86" t="s">
+        <v>288</v>
+      </c>
+      <c r="D86" t="s">
+        <v>289</v>
+      </c>
+      <c r="E86" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A87">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>331</v>
+        <v>291</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>332</v>
+        <v>292</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>333</v>
+        <v>293</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>334</v>
+        <v>294</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A88">
+        <v>74</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A89">
+        <v>75</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A90">
+        <v>76</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C90" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A91">
+        <v>77</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A92">
+        <v>78</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A93">
+        <v>79</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A94">
+        <v>80</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A95">
+        <v>81</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A96">
+        <v>82</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A97">
+        <v>83</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A98">
         <v>84</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B98" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A99">
+        <v>85</v>
+      </c>
+      <c r="B99" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="C88" s="3" t="s">
+      <c r="C99" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="D88" s="3" t="s">
+      <c r="D99" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="E88" s="6" t="s">
+      <c r="E99" s="6" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A89" s="9">
-        <v>85</v>
-      </c>
-      <c r="B89" s="3" t="s">
+    <row r="100" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A100">
+        <v>86</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C100" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="C89" s="3" t="s">
+      <c r="D100" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="D89" s="3" t="s">
+      <c r="E100" s="11" t="s">
         <v>395</v>
       </c>
-      <c r="E89" s="11" t="s">
+    </row>
+    <row r="101" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A101">
+        <v>87</v>
+      </c>
+      <c r="B101" s="3" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A90" s="9">
-        <v>86</v>
-      </c>
-      <c r="B90" s="3" t="s">
+      <c r="C101" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="C90" s="3" t="s">
+      <c r="D101" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="D90" s="3" t="s">
+      <c r="E101" s="10" t="s">
         <v>399</v>
       </c>
-      <c r="E90" s="10" t="s">
+    </row>
+    <row r="102" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A102">
+        <v>88</v>
+      </c>
+      <c r="B102" s="3" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A91" s="9">
-        <v>87</v>
-      </c>
-      <c r="B91" s="3" t="s">
+      <c r="C102" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="C91" s="3" t="s">
+      <c r="D102" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="D91" s="3" t="s">
+      <c r="E102" s="10" t="s">
         <v>403</v>
       </c>
-      <c r="E91" s="10" t="s">
+    </row>
+    <row r="103" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A103">
+        <v>89</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A92" s="9">
-        <v>88</v>
-      </c>
-      <c r="B92" s="3" t="s">
+      <c r="C103" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="D103" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="D92" s="3" t="s">
+      <c r="E103" s="10" t="s">
         <v>407</v>
       </c>
-      <c r="E92" s="10" t="s">
+    </row>
+    <row r="104" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A104" s="9">
+        <v>89</v>
+      </c>
+      <c r="B104" s="3"/>
+      <c r="C104" s="3" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A93" s="9">
-        <v>88</v>
-      </c>
-      <c r="B93" s="3"/>
-      <c r="C93" s="3" t="s">
+      <c r="D104" s="3"/>
+      <c r="E104" s="10"/>
+    </row>
+    <row r="105" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A105" s="9">
+        <v>90</v>
+      </c>
+      <c r="B105" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="C105" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="D93" s="3"/>
-      <c r="E93" s="10"/>
-    </row>
-    <row r="94" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" s="9">
-        <v>89</v>
-      </c>
-      <c r="B94" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="C94" s="9" t="s">
+      <c r="D105" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="D94" s="9" t="s">
+      <c r="E105" s="9" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A106" s="9">
+        <v>91</v>
+      </c>
+      <c r="B106" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="E94" s="9" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A95" s="9">
-        <v>90</v>
-      </c>
-      <c r="B95" s="9" t="s">
+      <c r="C106" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="D106" s="9" t="s">
         <v>412</v>
       </c>
-      <c r="C95" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="D95" s="9" t="s">
+      <c r="E106" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="E95" s="9" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A96" s="9">
-        <v>91</v>
-      </c>
-      <c r="B96" s="9" t="s">
+    </row>
+    <row r="107" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A107" s="9">
+        <v>92</v>
+      </c>
+      <c r="B107" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="C107" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="D107" s="9" t="s">
         <v>423</v>
       </c>
-      <c r="D96" s="9" t="s">
+      <c r="E107" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="E96" s="9" t="s">
+    </row>
+    <row r="108" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A108" s="9">
+        <v>93</v>
+      </c>
+      <c r="B108" s="9" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A97" s="9">
-        <v>92</v>
-      </c>
-      <c r="B97" s="9" t="s">
+      <c r="C108" s="9" t="s">
         <v>426</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="D108" s="9" t="s">
         <v>427</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="E108" s="9" t="s">
         <v>428</v>
       </c>
-      <c r="E97" s="9" t="s">
+    </row>
+    <row r="109" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A109" s="9">
+        <v>94</v>
+      </c>
+      <c r="B109" s="3" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A98" s="9">
-        <v>93</v>
-      </c>
-      <c r="B98" s="3" t="s">
+      <c r="C109" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="C98" s="3" t="s">
+      <c r="D109" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="D98" s="3" t="s">
+      <c r="E109" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="E98" s="10" t="s">
+    </row>
+    <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A110" s="9">
+        <v>95</v>
+      </c>
+      <c r="B110" s="9" t="s">
         <v>433</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A99" s="9">
-        <v>94</v>
-      </c>
-      <c r="B99" s="9" t="s">
+      <c r="C110" s="9" t="s">
         <v>434</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="D110" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="E110" s="9" t="s">
         <v>436</v>
       </c>
-      <c r="E99" s="9" t="s">
+    </row>
+    <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A111" s="9">
+        <v>96</v>
+      </c>
+      <c r="B111" s="9" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" s="9">
-        <v>95</v>
-      </c>
-      <c r="B100" s="9" t="s">
+      <c r="C111" s="9" t="s">
         <v>438</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="D111" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="E111" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="E100" s="9" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A101" s="9">
-        <v>96</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>397</v>
-      </c>
-      <c r="C101" s="9" t="s">
+    </row>
+    <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A112" s="9">
+        <v>97</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="D112" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="E112" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="D101" s="9" t="s">
-        <v>399</v>
-      </c>
-      <c r="E101" s="9" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A102" s="9">
-        <v>97</v>
-      </c>
-      <c r="B102" s="9" t="s">
+    </row>
+    <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A113" s="9">
+        <v>98</v>
+      </c>
+      <c r="B113" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="C113" s="9" t="s">
         <v>607</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="D113" s="9" t="s">
         <v>608</v>
       </c>
-      <c r="D102" s="9" t="s">
+      <c r="E113" s="9" t="s">
         <v>609</v>
       </c>
-      <c r="E102" s="9" t="s">
+    </row>
+    <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A114" s="9">
+        <v>99</v>
+      </c>
+      <c r="B114" s="9" t="s">
         <v>610</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A103" s="9">
-        <v>98</v>
-      </c>
-      <c r="B103" s="9" t="s">
+      <c r="C114" s="9" t="s">
         <v>611</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="D114" s="12" t="s">
         <v>612</v>
       </c>
-      <c r="D103" s="12" t="s">
+      <c r="E114" s="9" t="s">
         <v>613</v>
-      </c>
-      <c r="E103" s="9" t="s">
-        <v>614</v>
       </c>
     </row>
   </sheetData>
@@ -4041,7 +4154,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9878D5F-0194-4AC6-B566-F63E204E3C96}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.73046875" customWidth="1"/>
@@ -4169,7 +4282,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4177,27 +4290,27 @@
         <v>349</v>
       </c>
       <c r="C8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D8" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="E8" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C9" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D9" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E9" t="s">
         <v>353</v>
@@ -4211,13 +4324,13 @@
         <v>354</v>
       </c>
       <c r="C10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D10" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E10" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -4225,13 +4338,13 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C11" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D11" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E11" t="s">
         <v>358</v>
@@ -4262,102 +4375,83 @@
         <v>360</v>
       </c>
       <c r="C13" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D13" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E13" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
-      <c r="B14" t="s">
-        <v>361</v>
-      </c>
-      <c r="C14" t="s">
-        <v>362</v>
-      </c>
-      <c r="D14" t="s">
-        <v>363</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="B14" s="3" t="s">
         <v>364</v>
       </c>
+      <c r="C14" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D15" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>368</v>
+      <c r="B16" s="9" t="s">
+        <v>458</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>369</v>
+        <v>459</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A17" s="9">
+        <v>459</v>
+      </c>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="E17" s="10" t="s">
         <v>461</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A18" s="9">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="9">
-        <v>17</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>464</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4396,16 +4490,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C2" t="s">
         <v>371</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>372</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>373</v>
-      </c>
-      <c r="E2" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4413,7 +4507,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4421,16 +4515,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" t="s">
         <v>376</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>377</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>378</v>
-      </c>
-      <c r="E4" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4438,16 +4532,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>379</v>
+      </c>
+      <c r="C5" t="s">
         <v>380</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>381</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>382</v>
-      </c>
-      <c r="E5" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4455,7 +4549,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4463,16 +4557,16 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
+        <v>384</v>
+      </c>
+      <c r="C7" t="s">
         <v>385</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>386</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>387</v>
-      </c>
-      <c r="E7" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4480,16 +4574,16 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
+        <v>388</v>
+      </c>
+      <c r="C8" t="s">
         <v>389</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>390</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>391</v>
-      </c>
-      <c r="E8" t="s">
-        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -4524,7 +4618,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4532,7 +4626,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4540,7 +4634,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4548,16 +4642,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>459</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>460</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4565,7 +4659,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4573,7 +4667,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4581,7 +4675,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
   </sheetData>
@@ -4622,16 +4716,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>395</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4639,16 +4733,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>399</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4656,16 +4750,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>403</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4673,16 +4767,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="6" t="s">
         <v>407</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4691,7 +4785,7 @@
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="6"/>
@@ -4704,10 +4798,10 @@
         <v>329</v>
       </c>
       <c r="C7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D7" t="s">
         <v>410</v>
-      </c>
-      <c r="D7" t="s">
-        <v>411</v>
       </c>
       <c r="E7" t="s">
         <v>330</v>
@@ -4718,16 +4812,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
+        <v>411</v>
+      </c>
+      <c r="C8" t="s">
+        <v>411</v>
+      </c>
+      <c r="D8" t="s">
         <v>412</v>
       </c>
-      <c r="C8" t="s">
-        <v>412</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>413</v>
-      </c>
-      <c r="E8" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -4735,16 +4829,16 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>414</v>
+      </c>
+      <c r="C9" t="s">
         <v>415</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>416</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>417</v>
-      </c>
-      <c r="E9" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -4752,16 +4846,16 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
+        <v>418</v>
+      </c>
+      <c r="C10" t="s">
+        <v>418</v>
+      </c>
+      <c r="D10" t="s">
         <v>419</v>
       </c>
-      <c r="C10" t="s">
-        <v>419</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>420</v>
-      </c>
-      <c r="E10" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -4769,16 +4863,16 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
+        <v>421</v>
+      </c>
+      <c r="C11" t="s">
         <v>422</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>423</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>424</v>
-      </c>
-      <c r="E11" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4786,16 +4880,16 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
+        <v>425</v>
+      </c>
+      <c r="C12" t="s">
         <v>426</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>427</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>428</v>
-      </c>
-      <c r="E12" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -4803,16 +4897,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="6" t="s">
         <v>432</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -4820,16 +4914,16 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
+        <v>433</v>
+      </c>
+      <c r="C14" t="s">
         <v>434</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>435</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>436</v>
-      </c>
-      <c r="E14" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -4837,16 +4931,16 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
+        <v>437</v>
+      </c>
+      <c r="C15" t="s">
         <v>438</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>439</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>440</v>
-      </c>
-      <c r="E15" t="s">
-        <v>441</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -4854,16 +4948,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
+        <v>441</v>
+      </c>
+      <c r="C16" t="s">
         <v>442</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>443</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>444</v>
-      </c>
-      <c r="E16" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -4871,16 +4965,16 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C17" t="s">
+        <v>445</v>
+      </c>
+      <c r="D17" t="s">
+        <v>398</v>
+      </c>
+      <c r="E17" t="s">
         <v>446</v>
-      </c>
-      <c r="D17" t="s">
-        <v>399</v>
-      </c>
-      <c r="E17" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -4888,16 +4982,16 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
+        <v>447</v>
+      </c>
+      <c r="C18" t="s">
         <v>448</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>449</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>450</v>
-      </c>
-      <c r="E18" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -4905,16 +4999,16 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
+        <v>451</v>
+      </c>
+      <c r="C19" t="s">
         <v>452</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>453</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>454</v>
-      </c>
-      <c r="E19" t="s">
-        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -4955,16 +5049,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>464</v>
+      </c>
+      <c r="C2" t="s">
         <v>465</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>466</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>467</v>
-      </c>
-      <c r="E2" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4972,16 +5066,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>468</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" t="s">
         <v>470</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>471</v>
-      </c>
-      <c r="E3" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4989,16 +5083,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>472</v>
+      </c>
+      <c r="C4" t="s">
         <v>473</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>474</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>475</v>
-      </c>
-      <c r="E4" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5006,16 +5100,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C5" t="s">
         <v>477</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>478</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>479</v>
-      </c>
-      <c r="E5" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5023,16 +5117,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C6" t="s">
         <v>481</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>482</v>
       </c>
-      <c r="D6" t="s">
-        <v>483</v>
-      </c>
       <c r="E6" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5040,16 +5134,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>483</v>
+      </c>
+      <c r="C7" t="s">
         <v>484</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>485</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>486</v>
-      </c>
-      <c r="E7" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -5057,16 +5151,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
+        <v>487</v>
+      </c>
+      <c r="C8" t="s">
         <v>488</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>489</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>490</v>
-      </c>
-      <c r="E8" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -5074,16 +5168,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
+        <v>491</v>
+      </c>
+      <c r="C9" t="s">
         <v>492</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>493</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>494</v>
-      </c>
-      <c r="E9" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -5091,16 +5185,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
+        <v>495</v>
+      </c>
+      <c r="C10" t="s">
         <v>496</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>497</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>498</v>
-      </c>
-      <c r="E10" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -5108,16 +5202,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
+        <v>499</v>
+      </c>
+      <c r="C11" t="s">
         <v>500</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>501</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>502</v>
-      </c>
-      <c r="E11" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -5125,16 +5219,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
+        <v>503</v>
+      </c>
+      <c r="C12" t="s">
         <v>504</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>505</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>506</v>
-      </c>
-      <c r="E12" t="s">
-        <v>507</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -5142,16 +5236,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
+        <v>507</v>
+      </c>
+      <c r="C13" t="s">
         <v>508</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>509</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>510</v>
-      </c>
-      <c r="E13" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -5159,16 +5253,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
+        <v>511</v>
+      </c>
+      <c r="C14" t="s">
         <v>512</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>513</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>514</v>
-      </c>
-      <c r="E14" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -5176,16 +5270,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
+        <v>515</v>
+      </c>
+      <c r="C15" t="s">
         <v>516</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>517</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>518</v>
-      </c>
-      <c r="E15" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -5193,16 +5287,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
+        <v>519</v>
+      </c>
+      <c r="C16" t="s">
         <v>520</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>521</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>522</v>
-      </c>
-      <c r="E16" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -5210,16 +5304,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
+        <v>523</v>
+      </c>
+      <c r="C17" t="s">
         <v>524</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>525</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>526</v>
-      </c>
-      <c r="E17" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -5227,16 +5321,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
+        <v>527</v>
+      </c>
+      <c r="C18" t="s">
         <v>528</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>529</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>530</v>
-      </c>
-      <c r="E18" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -5244,16 +5338,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
+        <v>531</v>
+      </c>
+      <c r="C19" t="s">
         <v>532</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>533</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>534</v>
-      </c>
-      <c r="E19" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
@@ -5261,16 +5355,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
+        <v>535</v>
+      </c>
+      <c r="C20" t="s">
         <v>536</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>537</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>538</v>
-      </c>
-      <c r="E20" t="s">
-        <v>539</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
@@ -5278,16 +5372,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>539</v>
+      </c>
+      <c r="C21" t="s">
         <v>540</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>541</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>542</v>
-      </c>
-      <c r="E21" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
@@ -5295,16 +5389,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
+        <v>543</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>544</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>545</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" t="s">
         <v>546</v>
-      </c>
-      <c r="E22" t="s">
-        <v>547</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
@@ -5312,16 +5406,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
+        <v>547</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>549</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" t="s">
         <v>550</v>
-      </c>
-      <c r="E23" t="s">
-        <v>551</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -5329,16 +5423,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
+        <v>551</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>552</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>553</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="E24" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -5346,16 +5440,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>553</v>
+      </c>
+      <c r="C25" t="s">
         <v>554</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>555</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>556</v>
-      </c>
-      <c r="E25" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
@@ -5363,16 +5457,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
+        <v>557</v>
+      </c>
+      <c r="C26" t="s">
         <v>558</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>559</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>560</v>
-      </c>
-      <c r="E26" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
@@ -5380,16 +5474,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
+        <v>561</v>
+      </c>
+      <c r="C27" t="s">
         <v>562</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>563</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>564</v>
-      </c>
-      <c r="E27" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
@@ -5397,16 +5491,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
+        <v>565</v>
+      </c>
+      <c r="C28" t="s">
         <v>566</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>567</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>568</v>
-      </c>
-      <c r="E28" t="s">
-        <v>569</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
@@ -5414,16 +5508,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
+        <v>569</v>
+      </c>
+      <c r="C29" t="s">
         <v>570</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>571</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>572</v>
-      </c>
-      <c r="E29" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -5431,16 +5525,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
+        <v>573</v>
+      </c>
+      <c r="C30" t="s">
         <v>574</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>575</v>
       </c>
-      <c r="D30" t="s">
-        <v>576</v>
-      </c>
       <c r="E30" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
@@ -5448,16 +5542,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
+        <v>576</v>
+      </c>
+      <c r="C31" t="s">
         <v>577</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>578</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>579</v>
-      </c>
-      <c r="E31" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
@@ -5465,16 +5559,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
+        <v>580</v>
+      </c>
+      <c r="C32" t="s">
         <v>581</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>582</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>583</v>
-      </c>
-      <c r="E32" t="s">
-        <v>584</v>
       </c>
     </row>
   </sheetData>
@@ -5509,16 +5603,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>584</v>
+      </c>
+      <c r="C2" t="s">
         <v>585</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>585</v>
+      </c>
+      <c r="E2" t="s">
         <v>586</v>
-      </c>
-      <c r="D2" t="s">
-        <v>586</v>
-      </c>
-      <c r="E2" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -5526,16 +5620,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
+        <v>587</v>
+      </c>
+      <c r="C3" t="s">
         <v>588</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>589</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>590</v>
-      </c>
-      <c r="E3" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -5543,16 +5637,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>591</v>
+      </c>
+      <c r="C4" t="s">
         <v>592</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>593</v>
       </c>
-      <c r="D4" t="s">
-        <v>594</v>
-      </c>
       <c r="E4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5560,16 +5654,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>594</v>
+      </c>
+      <c r="C5" t="s">
         <v>595</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>596</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>597</v>
-      </c>
-      <c r="E5" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5577,16 +5671,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>598</v>
+      </c>
+      <c r="C6" t="s">
         <v>599</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>604</v>
+      </c>
+      <c r="E6" t="s">
         <v>600</v>
-      </c>
-      <c r="D6" t="s">
-        <v>605</v>
-      </c>
-      <c r="E6" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5594,16 +5688,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>601</v>
+      </c>
+      <c r="C7" t="s">
         <v>602</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>602</v>
+      </c>
+      <c r="E7" t="s">
         <v>603</v>
-      </c>
-      <c r="D7" t="s">
-        <v>603</v>
-      </c>
-      <c r="E7" t="s">
-        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -5612,17 +5706,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -5631,7 +5714,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -5892,18 +5975,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
-    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -5911,7 +5994,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5928,4 +6011,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
+    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
change to updated parquet file, classify additional 2023 data
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D05AEC-E955-4F41-AD84-8F72D54AC743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2352A72-8A63-4C9A-A328-5C7CCF363187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="626">
   <si>
     <t>id</t>
   </si>
@@ -1909,6 +1909,15 @@
   </si>
   <si>
     <t>death registration</t>
+  </si>
+  <si>
+    <t>death registry</t>
+  </si>
+  <si>
+    <t>vital register</t>
+  </si>
+  <si>
+    <t>vital registry</t>
   </si>
 </sst>
 </file>
@@ -2321,7 +2330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E114"/>
+  <dimension ref="A1:E117"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="24.1328125" customWidth="1"/>
@@ -2970,1179 +2979,1203 @@
         <v>32</v>
       </c>
       <c r="B42" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A43">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B43" t="s">
-        <v>135</v>
-      </c>
-      <c r="C43" t="s">
-        <v>136</v>
-      </c>
-      <c r="D43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E43" t="s">
-        <v>138</v>
+        <v>622</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A44">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B44" t="s">
-        <v>139</v>
+        <v>624</v>
       </c>
       <c r="C44" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D44" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E44" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A45">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B45" t="s">
-        <v>143</v>
-      </c>
-      <c r="C45" t="s">
-        <v>144</v>
-      </c>
-      <c r="D45" t="s">
-        <v>145</v>
-      </c>
-      <c r="E45" t="s">
-        <v>146</v>
+        <v>625</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A46">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
-      </c>
-      <c r="C46" t="s">
-        <v>148</v>
-      </c>
-      <c r="D46" t="s">
-        <v>149</v>
-      </c>
-      <c r="E46" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A47">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B47" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="C47" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D47" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="E47" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A48">
-        <v>37</v>
+        <v>35</v>
+      </c>
+      <c r="B48" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" t="s">
+        <v>144</v>
       </c>
       <c r="D48" t="s">
-        <v>155</v>
+        <v>145</v>
+      </c>
+      <c r="E48" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A49">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="D49" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="E49" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A50">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="B50" t="s">
+        <v>151</v>
+      </c>
+      <c r="C50" t="s">
+        <v>152</v>
       </c>
       <c r="D50" t="s">
-        <v>160</v>
+        <v>153</v>
+      </c>
+      <c r="E50" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A51">
-        <v>39</v>
-      </c>
-      <c r="B51" t="s">
-        <v>161</v>
-      </c>
-      <c r="C51" t="s">
-        <v>162</v>
+        <v>37</v>
       </c>
       <c r="D51" t="s">
-        <v>163</v>
-      </c>
-      <c r="E51" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A52">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B52" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="C52" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="D52" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="E52" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A53">
-        <v>41</v>
-      </c>
-      <c r="B53" t="s">
-        <v>169</v>
-      </c>
-      <c r="C53" t="s">
-        <v>170</v>
+        <v>38</v>
       </c>
       <c r="D53" t="s">
-        <v>171</v>
-      </c>
-      <c r="E53" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A54">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B54" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="C54" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D54" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E54" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A55">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B55" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="C55" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="D55" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E55" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A56">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B56" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="C56" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="D56" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="E56" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A57">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B57" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="C57" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="D57" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="E57" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A58">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B58" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="C58" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D58" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="E58" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A59">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="C59" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="D59" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="E59" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A60">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B60" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C60" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="D60" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="E60" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A61">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B61" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C61" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="D61" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="E61" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A62">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B62" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="C62" t="s">
         <v>194</v>
       </c>
       <c r="D62" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E62" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A63">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B63" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="C63" t="s">
         <v>198</v>
       </c>
       <c r="D63" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="E63" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A64">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B64" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C64" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="D64" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="E64" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A65">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B65" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C65" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="D65" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="E65" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A66">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B66" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="C66" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="D66" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="E66" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A67">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B67" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C67" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="D67" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="E67" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A68">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B68" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="C68" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="D68" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="E68" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A69">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B69" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="C69" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="D69" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="E69" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A70">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B70" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="C70" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="D70" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="E70" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A71">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B71" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="C71" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="D71" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="E71" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A72">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B72" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="C72" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="D72" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="E72" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A73">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B73" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="C73" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="D73" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="E73" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A74">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B74" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="C74" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="D74" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="E74" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A75">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B75" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="C75" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="D75" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="E75" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A76">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B76" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="C76" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="D76" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="E76" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A77">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B77" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="C77" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="D77" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
       <c r="E77" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A78">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B78" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="C78" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="D78" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="E78" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A79">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B79" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="C79" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="D79" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="E79" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A80">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B80" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="C80" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="D80" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="E80" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A81">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B81" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="C81" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="D81" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="E81" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A82">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B82" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="C82" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="D82" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="E82" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A83">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B83" t="s">
-        <v>52</v>
+        <v>275</v>
+      </c>
+      <c r="C83" t="s">
+        <v>276</v>
+      </c>
+      <c r="D83" t="s">
+        <v>277</v>
+      </c>
+      <c r="E83" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A84">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B84" t="s">
-        <v>621</v>
+        <v>279</v>
+      </c>
+      <c r="C84" t="s">
+        <v>280</v>
+      </c>
+      <c r="D84" t="s">
+        <v>281</v>
+      </c>
+      <c r="E84" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A85">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B85" t="s">
-        <v>617</v>
+        <v>283</v>
+      </c>
+      <c r="C85" t="s">
+        <v>284</v>
+      </c>
+      <c r="D85" t="s">
+        <v>285</v>
+      </c>
+      <c r="E85" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A86">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B86" t="s">
-        <v>287</v>
-      </c>
-      <c r="C86" t="s">
-        <v>288</v>
-      </c>
-      <c r="D86" t="s">
-        <v>289</v>
-      </c>
-      <c r="E86" t="s">
-        <v>290</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A87">
-        <v>73</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>294</v>
+        <v>71</v>
+      </c>
+      <c r="B87" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A88">
-        <v>74</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C88" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E88" s="6" t="s">
-        <v>298</v>
+        <v>71</v>
+      </c>
+      <c r="B88" t="s">
+        <v>617</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A89">
-        <v>75</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E89" s="6" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+        <v>72</v>
+      </c>
+      <c r="B89" t="s">
+        <v>287</v>
+      </c>
+      <c r="C89" t="s">
+        <v>288</v>
+      </c>
+      <c r="D89" t="s">
+        <v>289</v>
+      </c>
+      <c r="E89" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A90">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A91">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A92">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>316</v>
+        <v>303</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A94">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A95">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A96">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A97">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A98">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A99">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A100">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>392</v>
+        <v>329</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>393</v>
+        <v>329</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="E100" s="11" t="s">
-        <v>395</v>
+        <v>329</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A101">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>396</v>
+        <v>331</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>397</v>
+        <v>332</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="E101" s="10" t="s">
-        <v>399</v>
+        <v>333</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>334</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A102">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>400</v>
+        <v>335</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>401</v>
+        <v>336</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="E102" s="10" t="s">
-        <v>403</v>
+        <v>337</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A103">
+        <v>86</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="E103" s="11" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A104">
+        <v>87</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="E104" s="10" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A105">
+        <v>88</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="E105" s="10" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A106">
         <v>89</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B106" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="C106" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="D103" s="3" t="s">
+      <c r="D106" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="E103" s="10" t="s">
+      <c r="E106" s="10" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A104" s="9">
+    <row r="107" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A107" s="9">
         <v>89</v>
       </c>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3" t="s">
+      <c r="B107" s="3"/>
+      <c r="C107" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="D104" s="3"/>
-      <c r="E104" s="10"/>
-    </row>
-    <row r="105" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A105" s="9">
-        <v>90</v>
-      </c>
-      <c r="B105" s="9" t="s">
-        <v>329</v>
-      </c>
-      <c r="C105" s="9" t="s">
-        <v>409</v>
-      </c>
-      <c r="D105" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="E105" s="9" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A106" s="9">
-        <v>91</v>
-      </c>
-      <c r="B106" s="9" t="s">
-        <v>411</v>
-      </c>
-      <c r="C106" s="9" t="s">
-        <v>411</v>
-      </c>
-      <c r="D106" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="E106" s="9" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A107" s="9">
-        <v>92</v>
-      </c>
-      <c r="B107" s="9" t="s">
-        <v>421</v>
-      </c>
-      <c r="C107" s="9" t="s">
-        <v>422</v>
-      </c>
-      <c r="D107" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="E107" s="9" t="s">
-        <v>424</v>
-      </c>
+      <c r="D107" s="3"/>
+      <c r="E107" s="10"/>
     </row>
     <row r="108" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="9">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>425</v>
+        <v>329</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>426</v>
+        <v>409</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>427</v>
+        <v>410</v>
       </c>
       <c r="E108" s="9" t="s">
-        <v>428</v>
+        <v>330</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="9">
-        <v>94</v>
-      </c>
-      <c r="B109" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>430</v>
-      </c>
-      <c r="D109" s="3" t="s">
-        <v>431</v>
-      </c>
-      <c r="E109" s="10" t="s">
-        <v>432</v>
+        <v>91</v>
+      </c>
+      <c r="B109" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="C109" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="D109" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="E109" s="9" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="9">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="D110" s="9" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="E110" s="9" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" s="9">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" s="9">
-        <v>97</v>
-      </c>
-      <c r="B112" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="C112" s="9" t="s">
-        <v>445</v>
-      </c>
-      <c r="D112" s="9" t="s">
-        <v>398</v>
-      </c>
-      <c r="E112" s="9" t="s">
-        <v>446</v>
+        <v>94</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D112" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="E112" s="10" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" s="9">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>606</v>
+        <v>433</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>607</v>
+        <v>434</v>
       </c>
       <c r="D113" s="9" t="s">
-        <v>608</v>
+        <v>435</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>609</v>
+        <v>436</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" s="9">
+        <v>96</v>
+      </c>
+      <c r="B114" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="D114" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="E114" s="9" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A115" s="9">
+        <v>97</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="C115" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="D115" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="E115" s="9" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A116" s="9">
+        <v>98</v>
+      </c>
+      <c r="B116" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="C116" s="9" t="s">
+        <v>607</v>
+      </c>
+      <c r="D116" s="9" t="s">
+        <v>608</v>
+      </c>
+      <c r="E116" s="9" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A117" s="9">
         <v>99</v>
       </c>
-      <c r="B114" s="9" t="s">
+      <c r="B117" s="9" t="s">
         <v>610</v>
       </c>
-      <c r="C114" s="9" t="s">
+      <c r="C117" s="9" t="s">
         <v>611</v>
       </c>
-      <c r="D114" s="12" t="s">
+      <c r="D117" s="12" t="s">
         <v>612</v>
       </c>
-      <c r="E114" s="9" t="s">
+      <c r="E117" s="9" t="s">
         <v>613</v>
       </c>
     </row>
@@ -5715,6 +5748,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -5975,17 +6019,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
   <ds:schemaRefs>
@@ -5995,6 +6028,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
+    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6011,15 +6055,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
-    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated output dataset, added descriptions to remove for top funding projects, unrobust keywords removed
</commit_message>
<xml_diff>
--- a/data/keywords/review/keyword_review_modernization.xlsx
+++ b/data/keywords/review/keyword_review_modernization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2352A72-8A63-4C9A-A328-5C7CCF363187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256ACDB4-6080-4F14-9E67-70ABF5ACDCAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="626">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="615">
   <si>
     <t>id</t>
   </si>
@@ -1071,15 +1071,6 @@
     <t>crvs</t>
   </si>
   <si>
-    <t>cpi</t>
-  </si>
-  <si>
-    <t>IPC</t>
-  </si>
-  <si>
-    <t>VPI</t>
-  </si>
-  <si>
     <t>d4d</t>
   </si>
   <si>
@@ -1125,31 +1116,7 @@
     <t xml:space="preserve">lfs </t>
   </si>
   <si>
-    <t>ETF</t>
-  </si>
-  <si>
-    <t>epa</t>
-  </si>
-  <si>
-    <t>AKE</t>
-  </si>
-  <si>
     <t>NSO</t>
-  </si>
-  <si>
-    <t>INS</t>
-  </si>
-  <si>
-    <t>INE</t>
-  </si>
-  <si>
-    <t>NSS</t>
-  </si>
-  <si>
-    <t>SSN</t>
-  </si>
-  <si>
-    <t>SEN</t>
   </si>
   <si>
     <t>landmine</t>
@@ -1966,12 +1933,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="9" tint="-0.499984740745262"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2005,6 +1974,7 @@
       <sz val="11"/>
       <color rgb="FF375623"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2463,7 +2433,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>615</v>
+        <v>604</v>
       </c>
       <c r="C8" t="s">
         <v>29</v>
@@ -2480,7 +2450,7 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>618</v>
+        <v>607</v>
       </c>
       <c r="E9" s="8"/>
     </row>
@@ -2514,7 +2484,7 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>619</v>
+        <v>608</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2522,7 +2492,7 @@
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>616</v>
+        <v>605</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2606,7 +2576,7 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>620</v>
+        <v>609</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2614,7 +2584,7 @@
         <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>614</v>
+        <v>603</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2979,7 +2949,7 @@
         <v>32</v>
       </c>
       <c r="B42" t="s">
-        <v>623</v>
+        <v>612</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2987,7 +2957,7 @@
         <v>32</v>
       </c>
       <c r="B43" t="s">
-        <v>622</v>
+        <v>611</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2995,7 +2965,7 @@
         <v>33</v>
       </c>
       <c r="B44" t="s">
-        <v>624</v>
+        <v>613</v>
       </c>
       <c r="C44" t="s">
         <v>136</v>
@@ -3012,7 +2982,7 @@
         <v>33</v>
       </c>
       <c r="B45" t="s">
-        <v>625</v>
+        <v>614</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3681,7 +3651,7 @@
         <v>71</v>
       </c>
       <c r="B87" t="s">
-        <v>621</v>
+        <v>610</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3689,7 +3659,7 @@
         <v>71</v>
       </c>
       <c r="B88" t="s">
-        <v>617</v>
+        <v>606</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3935,16 +3905,16 @@
         <v>86</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="E103" s="11" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3952,16 +3922,16 @@
         <v>87</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="E104" s="10" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3969,16 +3939,16 @@
         <v>88</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -3986,16 +3956,16 @@
         <v>89</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="E106" s="10" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -4004,7 +3974,7 @@
       </c>
       <c r="B107" s="3"/>
       <c r="C107" s="3" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" s="10"/>
@@ -4017,10 +3987,10 @@
         <v>329</v>
       </c>
       <c r="C108" s="9" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="E108" s="9" t="s">
         <v>330</v>
@@ -4031,16 +4001,16 @@
         <v>91</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="C109" s="9" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="D109" s="9" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="E109" s="9" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4048,16 +4018,16 @@
         <v>92</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="D110" s="9" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="E110" s="9" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4065,16 +4035,16 @@
         <v>93</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="E111" s="9" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4082,16 +4052,16 @@
         <v>94</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
       <c r="E112" s="10" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4099,16 +4069,16 @@
         <v>95</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="D113" s="9" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="E113" s="9" t="s">
-        <v>436</v>
+        <v>425</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4116,16 +4086,16 @@
         <v>96</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="C114" s="9" t="s">
-        <v>438</v>
+        <v>427</v>
       </c>
       <c r="D114" s="9" t="s">
-        <v>439</v>
+        <v>428</v>
       </c>
       <c r="E114" s="9" t="s">
-        <v>440</v>
+        <v>429</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4133,16 +4103,16 @@
         <v>97</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C115" s="9" t="s">
-        <v>445</v>
+        <v>434</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="E115" s="9" t="s">
-        <v>446</v>
+        <v>435</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4150,16 +4120,16 @@
         <v>98</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>606</v>
+        <v>595</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>607</v>
+        <v>596</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>608</v>
+        <v>597</v>
       </c>
       <c r="E116" s="9" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
@@ -4167,16 +4137,16 @@
         <v>99</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>610</v>
+        <v>599</v>
       </c>
       <c r="C117" s="9" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="D117" s="12" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
       <c r="E117" s="9" t="s">
-        <v>613</v>
+        <v>602</v>
       </c>
     </row>
   </sheetData>
@@ -4187,7 +4157,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9878D5F-0194-4AC6-B566-F63E204E3C96}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.73046875" customWidth="1"/>
@@ -4255,13 +4225,13 @@
         <v>343</v>
       </c>
       <c r="C4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4269,16 +4239,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E5" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4286,50 +4256,50 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="E6" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D7" t="s">
         <v>348</v>
       </c>
       <c r="E7" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C8" t="s">
         <v>350</v>
       </c>
       <c r="D8" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -4337,16 +4307,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C9" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D9" t="s">
         <v>353</v>
       </c>
       <c r="E9" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -4354,16 +4324,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C10" t="s">
         <v>355</v>
       </c>
       <c r="D10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E10" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -4371,16 +4341,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C11" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D11" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="E11" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4388,103 +4358,56 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>359</v>
-      </c>
-      <c r="C12" t="s">
-        <v>359</v>
-      </c>
-      <c r="D12" t="s">
-        <v>359</v>
-      </c>
-      <c r="E12" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>360</v>
-      </c>
-      <c r="C13" t="s">
-        <v>361</v>
-      </c>
-      <c r="D13" t="s">
-        <v>362</v>
-      </c>
-      <c r="E13" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B13" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>364</v>
+      <c r="B14" s="9" t="s">
+        <v>447</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>365</v>
+        <v>448</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+        <v>448</v>
+      </c>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="B15" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="E16" s="10"/>
-    </row>
-    <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A17">
-        <v>15</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>461</v>
-      </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-    </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18">
-        <v>16</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>463</v>
-      </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
+        <v>452</v>
+      </c>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4523,16 +4446,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="C2" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="D2" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="E2" t="s">
-        <v>373</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4540,7 +4463,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4548,16 +4471,16 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="C4" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="D4" t="s">
-        <v>377</v>
+        <v>366</v>
       </c>
       <c r="E4" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4565,16 +4488,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="C5" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="D5" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="E5" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4582,7 +4505,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>383</v>
+        <v>372</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4590,16 +4513,16 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>384</v>
+        <v>373</v>
       </c>
       <c r="C7" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="D7" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="E7" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4607,16 +4530,16 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="C8" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="D8" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="E8" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -4651,7 +4574,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>455</v>
+        <v>444</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4659,7 +4582,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4667,7 +4590,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>457</v>
+        <v>446</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4675,16 +4598,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>458</v>
+        <v>447</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>459</v>
+        <v>448</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>459</v>
+        <v>448</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>460</v>
+        <v>449</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4692,7 +4615,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>461</v>
+        <v>450</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -4700,7 +4623,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>462</v>
+        <v>451</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -4708,7 +4631,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>463</v>
+        <v>452</v>
       </c>
     </row>
   </sheetData>
@@ -4749,16 +4672,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -4766,16 +4689,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -4783,16 +4706,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -4800,16 +4723,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -4818,7 +4741,7 @@
       </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="6"/>
@@ -4831,10 +4754,10 @@
         <v>329</v>
       </c>
       <c r="C7" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="D7" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="E7" t="s">
         <v>330</v>
@@ -4845,16 +4768,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="C8" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="D8" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="E8" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -4862,16 +4785,16 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="C9" t="s">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="D9" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="E9" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -4879,16 +4802,16 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="C10" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="D10" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="E10" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -4896,16 +4819,16 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="C11" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="D11" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="E11" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -4913,16 +4836,16 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="C12" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="D12" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="E12" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -4930,16 +4853,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -4947,16 +4870,16 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="C14" t="s">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="D14" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="E14" t="s">
-        <v>436</v>
+        <v>425</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -4964,16 +4887,16 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="C15" t="s">
-        <v>438</v>
+        <v>427</v>
       </c>
       <c r="D15" t="s">
-        <v>439</v>
+        <v>428</v>
       </c>
       <c r="E15" t="s">
-        <v>440</v>
+        <v>429</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -4981,16 +4904,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>441</v>
+        <v>430</v>
       </c>
       <c r="C16" t="s">
-        <v>442</v>
+        <v>431</v>
       </c>
       <c r="D16" t="s">
-        <v>443</v>
+        <v>432</v>
       </c>
       <c r="E16" t="s">
-        <v>444</v>
+        <v>433</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -4998,16 +4921,16 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="C17" t="s">
-        <v>445</v>
+        <v>434</v>
       </c>
       <c r="D17" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="E17" t="s">
-        <v>446</v>
+        <v>435</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -5015,16 +4938,16 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>447</v>
+        <v>436</v>
       </c>
       <c r="C18" t="s">
-        <v>448</v>
+        <v>437</v>
       </c>
       <c r="D18" t="s">
-        <v>449</v>
+        <v>438</v>
       </c>
       <c r="E18" t="s">
-        <v>450</v>
+        <v>439</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -5032,16 +4955,16 @@
         <v>16</v>
       </c>
       <c r="B19" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="C19" t="s">
-        <v>452</v>
+        <v>441</v>
       </c>
       <c r="D19" t="s">
-        <v>453</v>
+        <v>442</v>
       </c>
       <c r="E19" t="s">
-        <v>454</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -5082,16 +5005,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>464</v>
+        <v>453</v>
       </c>
       <c r="C2" t="s">
-        <v>465</v>
+        <v>454</v>
       </c>
       <c r="D2" t="s">
-        <v>466</v>
+        <v>455</v>
       </c>
       <c r="E2" t="s">
-        <v>467</v>
+        <v>456</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -5099,16 +5022,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>468</v>
+        <v>457</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>469</v>
+        <v>458</v>
       </c>
       <c r="D3" t="s">
-        <v>470</v>
+        <v>459</v>
       </c>
       <c r="E3" t="s">
-        <v>471</v>
+        <v>460</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -5116,16 +5039,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>472</v>
+        <v>461</v>
       </c>
       <c r="C4" t="s">
-        <v>473</v>
+        <v>462</v>
       </c>
       <c r="D4" t="s">
-        <v>474</v>
+        <v>463</v>
       </c>
       <c r="E4" t="s">
-        <v>475</v>
+        <v>464</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5133,16 +5056,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>476</v>
+        <v>465</v>
       </c>
       <c r="C5" t="s">
-        <v>477</v>
+        <v>466</v>
       </c>
       <c r="D5" t="s">
-        <v>478</v>
+        <v>467</v>
       </c>
       <c r="E5" t="s">
-        <v>479</v>
+        <v>468</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5150,16 +5073,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>480</v>
+        <v>469</v>
       </c>
       <c r="C6" t="s">
-        <v>481</v>
+        <v>470</v>
       </c>
       <c r="D6" t="s">
-        <v>482</v>
+        <v>471</v>
       </c>
       <c r="E6" t="s">
-        <v>605</v>
+        <v>594</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5167,16 +5090,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>483</v>
+        <v>472</v>
       </c>
       <c r="C7" t="s">
-        <v>484</v>
+        <v>473</v>
       </c>
       <c r="D7" t="s">
-        <v>485</v>
+        <v>474</v>
       </c>
       <c r="E7" t="s">
-        <v>486</v>
+        <v>475</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -5184,16 +5107,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>487</v>
+        <v>476</v>
       </c>
       <c r="C8" t="s">
-        <v>488</v>
+        <v>477</v>
       </c>
       <c r="D8" t="s">
-        <v>489</v>
+        <v>478</v>
       </c>
       <c r="E8" t="s">
-        <v>490</v>
+        <v>479</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
@@ -5201,16 +5124,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>491</v>
+        <v>480</v>
       </c>
       <c r="C9" t="s">
-        <v>492</v>
+        <v>481</v>
       </c>
       <c r="D9" t="s">
-        <v>493</v>
+        <v>482</v>
       </c>
       <c r="E9" t="s">
-        <v>494</v>
+        <v>483</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.45">
@@ -5218,16 +5141,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>495</v>
+        <v>484</v>
       </c>
       <c r="C10" t="s">
-        <v>496</v>
+        <v>485</v>
       </c>
       <c r="D10" t="s">
-        <v>497</v>
+        <v>486</v>
       </c>
       <c r="E10" t="s">
-        <v>498</v>
+        <v>487</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.45">
@@ -5235,16 +5158,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>499</v>
+        <v>488</v>
       </c>
       <c r="C11" t="s">
-        <v>500</v>
+        <v>489</v>
       </c>
       <c r="D11" t="s">
-        <v>501</v>
+        <v>490</v>
       </c>
       <c r="E11" t="s">
-        <v>502</v>
+        <v>491</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.45">
@@ -5252,16 +5175,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>503</v>
+        <v>492</v>
       </c>
       <c r="C12" t="s">
-        <v>504</v>
+        <v>493</v>
       </c>
       <c r="D12" t="s">
-        <v>505</v>
+        <v>494</v>
       </c>
       <c r="E12" t="s">
-        <v>506</v>
+        <v>495</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.45">
@@ -5269,16 +5192,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>507</v>
+        <v>496</v>
       </c>
       <c r="C13" t="s">
-        <v>508</v>
+        <v>497</v>
       </c>
       <c r="D13" t="s">
-        <v>509</v>
+        <v>498</v>
       </c>
       <c r="E13" t="s">
-        <v>510</v>
+        <v>499</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.45">
@@ -5286,16 +5209,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>511</v>
+        <v>500</v>
       </c>
       <c r="C14" t="s">
-        <v>512</v>
+        <v>501</v>
       </c>
       <c r="D14" t="s">
-        <v>513</v>
+        <v>502</v>
       </c>
       <c r="E14" t="s">
-        <v>514</v>
+        <v>503</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.45">
@@ -5303,16 +5226,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>515</v>
+        <v>504</v>
       </c>
       <c r="C15" t="s">
-        <v>516</v>
+        <v>505</v>
       </c>
       <c r="D15" t="s">
-        <v>517</v>
+        <v>506</v>
       </c>
       <c r="E15" t="s">
-        <v>518</v>
+        <v>507</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.45">
@@ -5320,16 +5243,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>519</v>
+        <v>508</v>
       </c>
       <c r="C16" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="D16" t="s">
-        <v>521</v>
+        <v>510</v>
       </c>
       <c r="E16" t="s">
-        <v>522</v>
+        <v>511</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
@@ -5337,16 +5260,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="C17" t="s">
-        <v>524</v>
+        <v>513</v>
       </c>
       <c r="D17" t="s">
-        <v>525</v>
+        <v>514</v>
       </c>
       <c r="E17" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
@@ -5354,16 +5277,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>527</v>
+        <v>516</v>
       </c>
       <c r="C18" t="s">
-        <v>528</v>
+        <v>517</v>
       </c>
       <c r="D18" t="s">
-        <v>529</v>
+        <v>518</v>
       </c>
       <c r="E18" t="s">
-        <v>530</v>
+        <v>519</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
@@ -5371,16 +5294,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>531</v>
+        <v>520</v>
       </c>
       <c r="C19" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
       <c r="D19" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
       <c r="E19" t="s">
-        <v>534</v>
+        <v>523</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
@@ -5388,16 +5311,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
       <c r="C20" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
       <c r="D20" t="s">
-        <v>537</v>
+        <v>526</v>
       </c>
       <c r="E20" t="s">
-        <v>538</v>
+        <v>527</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
@@ -5405,16 +5328,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>539</v>
+        <v>528</v>
       </c>
       <c r="C21" t="s">
-        <v>540</v>
+        <v>529</v>
       </c>
       <c r="D21" t="s">
-        <v>541</v>
+        <v>530</v>
       </c>
       <c r="E21" t="s">
-        <v>542</v>
+        <v>531</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
@@ -5422,16 +5345,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>543</v>
+        <v>532</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>544</v>
+        <v>533</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>545</v>
+        <v>534</v>
       </c>
       <c r="E22" t="s">
-        <v>546</v>
+        <v>535</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
@@ -5439,16 +5362,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>547</v>
+        <v>536</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>548</v>
+        <v>537</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>549</v>
+        <v>538</v>
       </c>
       <c r="E23" t="s">
-        <v>550</v>
+        <v>539</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
@@ -5456,16 +5379,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>551</v>
+        <v>540</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>552</v>
+        <v>541</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>551</v>
+        <v>540</v>
       </c>
       <c r="E24" t="s">
-        <v>551</v>
+        <v>540</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
@@ -5473,16 +5396,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>553</v>
+        <v>542</v>
       </c>
       <c r="C25" t="s">
-        <v>554</v>
+        <v>543</v>
       </c>
       <c r="D25" t="s">
-        <v>555</v>
+        <v>544</v>
       </c>
       <c r="E25" t="s">
-        <v>556</v>
+        <v>545</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
@@ -5490,16 +5413,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>557</v>
+        <v>546</v>
       </c>
       <c r="C26" t="s">
-        <v>558</v>
+        <v>547</v>
       </c>
       <c r="D26" t="s">
-        <v>559</v>
+        <v>548</v>
       </c>
       <c r="E26" t="s">
-        <v>560</v>
+        <v>549</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
@@ -5507,16 +5430,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>561</v>
+        <v>550</v>
       </c>
       <c r="C27" t="s">
-        <v>562</v>
+        <v>551</v>
       </c>
       <c r="D27" t="s">
-        <v>563</v>
+        <v>552</v>
       </c>
       <c r="E27" t="s">
-        <v>564</v>
+        <v>553</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
@@ -5524,16 +5447,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>565</v>
+        <v>554</v>
       </c>
       <c r="C28" t="s">
-        <v>566</v>
+        <v>555</v>
       </c>
       <c r="D28" t="s">
-        <v>567</v>
+        <v>556</v>
       </c>
       <c r="E28" t="s">
-        <v>568</v>
+        <v>557</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
@@ -5541,16 +5464,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>569</v>
+        <v>558</v>
       </c>
       <c r="C29" t="s">
-        <v>570</v>
+        <v>559</v>
       </c>
       <c r="D29" t="s">
-        <v>571</v>
+        <v>560</v>
       </c>
       <c r="E29" t="s">
-        <v>572</v>
+        <v>561</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
@@ -5558,16 +5481,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>573</v>
+        <v>562</v>
       </c>
       <c r="C30" t="s">
-        <v>574</v>
+        <v>563</v>
       </c>
       <c r="D30" t="s">
-        <v>575</v>
+        <v>564</v>
       </c>
       <c r="E30" t="s">
-        <v>514</v>
+        <v>503</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
@@ -5575,16 +5498,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>576</v>
+        <v>565</v>
       </c>
       <c r="C31" t="s">
-        <v>577</v>
+        <v>566</v>
       </c>
       <c r="D31" t="s">
-        <v>578</v>
+        <v>567</v>
       </c>
       <c r="E31" t="s">
-        <v>579</v>
+        <v>568</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
@@ -5592,16 +5515,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>580</v>
+        <v>569</v>
       </c>
       <c r="C32" t="s">
-        <v>581</v>
+        <v>570</v>
       </c>
       <c r="D32" t="s">
-        <v>582</v>
+        <v>571</v>
       </c>
       <c r="E32" t="s">
-        <v>583</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>
@@ -5636,16 +5559,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>584</v>
+        <v>573</v>
       </c>
       <c r="C2" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
       <c r="D2" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
       <c r="E2" t="s">
-        <v>586</v>
+        <v>575</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
@@ -5653,16 +5576,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>587</v>
+        <v>576</v>
       </c>
       <c r="C3" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
       <c r="D3" t="s">
-        <v>589</v>
+        <v>578</v>
       </c>
       <c r="E3" t="s">
-        <v>590</v>
+        <v>579</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
@@ -5670,16 +5593,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>591</v>
+        <v>580</v>
       </c>
       <c r="C4" t="s">
-        <v>592</v>
+        <v>581</v>
       </c>
       <c r="D4" t="s">
-        <v>593</v>
+        <v>582</v>
       </c>
       <c r="E4" t="s">
-        <v>591</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
@@ -5687,16 +5610,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>594</v>
+        <v>583</v>
       </c>
       <c r="C5" t="s">
-        <v>595</v>
+        <v>584</v>
       </c>
       <c r="D5" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
       <c r="E5" t="s">
-        <v>597</v>
+        <v>586</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -5704,16 +5627,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>598</v>
+        <v>587</v>
       </c>
       <c r="C6" t="s">
-        <v>599</v>
+        <v>588</v>
       </c>
       <c r="D6" t="s">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="E6" t="s">
-        <v>600</v>
+        <v>589</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
@@ -5721,16 +5644,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>601</v>
+        <v>590</v>
       </c>
       <c r="C7" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="D7" t="s">
-        <v>602</v>
+        <v>591</v>
       </c>
       <c r="E7" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
     </row>
   </sheetData>
@@ -5739,26 +5662,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -6019,10 +5922,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9bae65c2-241c-418a-a37c-ddfb2f921707" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
+    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6039,20 +5973,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
-    <ds:schemaRef ds:uri="9bae65c2-241c-418a-a37c-ddfb2f921707"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>